<commit_message>
Sutvarkyti pilni pavadinimai Greitis lape, nuimti suliejimai
</commit_message>
<xml_diff>
--- a/Ivestis.xlsx
+++ b/Ivestis.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr codeName="Šios_darbaknygės" defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://agentura2020-my.sharepoint.com/personal/sigitas_cekanauskas_gamta_lt/Documents/Dokumentai/STACIONARUS ORO TARSOS SALTINIAI/2026 m/Skaiciuokles KD, GR/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://agentura2020.sharepoint.com/sites/VidurioLietuvosaplinkostyrimuskyrius/Bendrai naudojami dokumentai/EB7-014 Darbuotojų failai/Tomo/Python 3.14.3/Skaiciavimai/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="262" documentId="13_ncr:1_{D8ED3FA4-1188-4E70-924F-660A50F19C4F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{ED64DD58-D285-4600-9422-E0BE97374520}"/>
+  <xr:revisionPtr revIDLastSave="263" documentId="13_ncr:1_{D8ED3FA4-1188-4E70-924F-660A50F19C4F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8685D0F3-FD86-4775-8711-4CB6F11BBCB9}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="821" firstSheet="1" activeTab="1" xr2:uid="{B097D0E3-85A4-46F7-964F-ABE00A6941B9}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" tabRatio="821" firstSheet="1" activeTab="1" xr2:uid="{B097D0E3-85A4-46F7-964F-ABE00A6941B9}"/>
   </bookViews>
   <sheets>
     <sheet name="Compatibility Report" sheetId="4" state="hidden" r:id="rId1"/>
@@ -2665,6 +2665,9 @@
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="164" fontId="4" fillId="2" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="49" fontId="10" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
       <protection locked="0"/>
@@ -2677,12 +2680,40 @@
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="14" fontId="30" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top"/>
+      <protection locked="0"/>
+    </xf>
     <xf numFmtId="0" fontId="30" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="center" vertical="top"/>
       <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="30" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="center" vertical="top"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
       <protection locked="0"/>
     </xf>
     <xf numFmtId="2" fontId="9" fillId="8" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
@@ -2705,6 +2736,14 @@
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
@@ -2768,6 +2807,42 @@
     <xf numFmtId="169" fontId="4" fillId="2" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="7" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
@@ -2785,83 +2860,8 @@
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="7" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="2" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="30" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
       <protection locked="0"/>
     </xf>
   </cellXfs>
@@ -3173,16 +3173,16 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1ABD58BE-2006-42BB-8F0B-A2F613982E7B}">
   <sheetPr codeName="Lapas1"/>
   <dimension ref="B1:E10"/>
-  <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultRowHeight="12.5" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="1.140625" customWidth="1"/>
-    <col min="2" max="2" width="64.42578125" customWidth="1"/>
-    <col min="3" max="3" width="1.5703125" customWidth="1"/>
-    <col min="4" max="4" width="5.5703125" customWidth="1"/>
+    <col min="1" max="1" width="1.1796875" customWidth="1"/>
+    <col min="2" max="2" width="64.453125" customWidth="1"/>
+    <col min="3" max="3" width="1.54296875" customWidth="1"/>
+    <col min="4" max="4" width="5.54296875" customWidth="1"/>
     <col min="5" max="5" width="16" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:5" x14ac:dyDescent="0.2">
+    <row r="1" spans="2:5" ht="13" x14ac:dyDescent="0.25">
       <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3190,7 +3190,7 @@
       <c r="D1" s="5"/>
       <c r="E1" s="5"/>
     </row>
-    <row r="2" spans="2:5" x14ac:dyDescent="0.2">
+    <row r="2" spans="2:5" ht="13" x14ac:dyDescent="0.25">
       <c r="B2" s="1" t="s">
         <v>1</v>
       </c>
@@ -3198,13 +3198,13 @@
       <c r="D2" s="5"/>
       <c r="E2" s="5"/>
     </row>
-    <row r="3" spans="2:5" x14ac:dyDescent="0.2">
+    <row r="3" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B3" s="2"/>
       <c r="C3" s="2"/>
       <c r="D3" s="6"/>
       <c r="E3" s="6"/>
     </row>
-    <row r="4" spans="2:5" ht="38.25" x14ac:dyDescent="0.2">
+    <row r="4" spans="2:5" ht="37.5" x14ac:dyDescent="0.25">
       <c r="B4" s="2" t="s">
         <v>2</v>
       </c>
@@ -3212,13 +3212,13 @@
       <c r="D4" s="6"/>
       <c r="E4" s="6"/>
     </row>
-    <row r="5" spans="2:5" x14ac:dyDescent="0.2">
+    <row r="5" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B5" s="2"/>
       <c r="C5" s="2"/>
       <c r="D5" s="6"/>
       <c r="E5" s="6"/>
     </row>
-    <row r="6" spans="2:5" x14ac:dyDescent="0.2">
+    <row r="6" spans="2:5" ht="13" x14ac:dyDescent="0.25">
       <c r="B6" s="1" t="s">
         <v>3</v>
       </c>
@@ -3228,13 +3228,13 @@
         <v>4</v>
       </c>
     </row>
-    <row r="7" spans="2:5" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:5" ht="13" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
       <c r="D7" s="6"/>
       <c r="E7" s="6"/>
     </row>
-    <row r="8" spans="2:5" ht="39" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="2:5" ht="38" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B8" s="3" t="s">
         <v>5</v>
       </c>
@@ -3244,13 +3244,13 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="2:5" x14ac:dyDescent="0.2">
+    <row r="9" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B9" s="2"/>
       <c r="C9" s="2"/>
       <c r="D9" s="6"/>
       <c r="E9" s="6"/>
     </row>
-    <row r="10" spans="2:5" x14ac:dyDescent="0.2">
+    <row r="10" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B10" s="2"/>
       <c r="C10" s="2"/>
       <c r="D10" s="6"/>
@@ -3265,61 +3265,61 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2678AA73-39E5-446A-B7DA-8D6634C4EC86}">
   <dimension ref="A2:AB26"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="15.5" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="2" width="11.28515625" style="171" customWidth="1"/>
-    <col min="3" max="3" width="15.85546875" style="171" customWidth="1"/>
-    <col min="4" max="4" width="9.85546875" style="171" customWidth="1"/>
-    <col min="5" max="5" width="11.5703125" style="171" customWidth="1"/>
-    <col min="6" max="6" width="11.42578125" style="171" customWidth="1"/>
-    <col min="7" max="7" width="10.5703125" style="171" customWidth="1"/>
-    <col min="8" max="12" width="9.140625" style="171"/>
-    <col min="13" max="13" width="11.140625" style="171" customWidth="1"/>
-    <col min="14" max="14" width="11.42578125" style="171" customWidth="1"/>
-    <col min="15" max="15" width="9.140625" style="171"/>
-    <col min="16" max="16" width="10.5703125" style="171" customWidth="1"/>
-    <col min="17" max="17" width="9.5703125" style="171" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="9.140625" style="171"/>
-    <col min="19" max="19" width="11.28515625" style="171" customWidth="1"/>
-    <col min="20" max="20" width="11.7109375" style="171" customWidth="1"/>
+    <col min="1" max="2" width="11.26953125" style="171" customWidth="1"/>
+    <col min="3" max="3" width="15.81640625" style="171" customWidth="1"/>
+    <col min="4" max="4" width="9.81640625" style="171" customWidth="1"/>
+    <col min="5" max="5" width="11.54296875" style="171" customWidth="1"/>
+    <col min="6" max="6" width="11.453125" style="171" customWidth="1"/>
+    <col min="7" max="7" width="10.54296875" style="171" customWidth="1"/>
+    <col min="8" max="12" width="9.1796875" style="171"/>
+    <col min="13" max="13" width="11.1796875" style="171" customWidth="1"/>
+    <col min="14" max="14" width="11.453125" style="171" customWidth="1"/>
+    <col min="15" max="15" width="9.1796875" style="171"/>
+    <col min="16" max="16" width="10.54296875" style="171" customWidth="1"/>
+    <col min="17" max="17" width="9.54296875" style="171" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="9.1796875" style="171"/>
+    <col min="19" max="19" width="11.26953125" style="171" customWidth="1"/>
+    <col min="20" max="20" width="11.7265625" style="171" customWidth="1"/>
     <col min="21" max="21" width="10" style="171" customWidth="1"/>
-    <col min="22" max="22" width="11.7109375" style="171" customWidth="1"/>
-    <col min="23" max="23" width="11.42578125" style="171" customWidth="1"/>
-    <col min="24" max="24" width="9.5703125" style="171" customWidth="1"/>
-    <col min="25" max="26" width="10.28515625" style="171" customWidth="1"/>
-    <col min="27" max="27" width="9.140625" style="171"/>
-    <col min="28" max="28" width="10.7109375" style="171" customWidth="1"/>
-    <col min="29" max="16384" width="9.140625" style="171"/>
+    <col min="22" max="22" width="11.7265625" style="171" customWidth="1"/>
+    <col min="23" max="23" width="11.453125" style="171" customWidth="1"/>
+    <col min="24" max="24" width="9.54296875" style="171" customWidth="1"/>
+    <col min="25" max="26" width="10.26953125" style="171" customWidth="1"/>
+    <col min="27" max="27" width="9.1796875" style="171"/>
+    <col min="28" max="28" width="10.7265625" style="171" customWidth="1"/>
+    <col min="29" max="16384" width="9.1796875" style="171"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:28" x14ac:dyDescent="0.2">
-      <c r="D2" s="244" t="s">
+    <row r="2" spans="1:28" x14ac:dyDescent="0.25">
+      <c r="D2" s="245" t="s">
         <v>108</v>
       </c>
-      <c r="E2" s="244"/>
-      <c r="F2" s="244"/>
-      <c r="G2" s="244"/>
-      <c r="H2" s="244"/>
-      <c r="I2" s="244"/>
-      <c r="J2" s="244"/>
-      <c r="K2" s="244"/>
-      <c r="L2" s="244"/>
-      <c r="M2" s="244"/>
-      <c r="N2" s="244"/>
-      <c r="O2" s="244"/>
-      <c r="P2" s="244"/>
-      <c r="Q2" s="244"/>
-      <c r="R2" s="244"/>
-      <c r="S2" s="244"/>
-      <c r="T2" s="244"/>
-      <c r="U2" s="244"/>
-      <c r="V2" s="244"/>
-      <c r="W2" s="244"/>
-      <c r="X2" s="244"/>
-      <c r="Y2" s="244"/>
-      <c r="Z2" s="244"/>
-    </row>
-    <row r="4" spans="1:28" s="10" customFormat="1" ht="150" x14ac:dyDescent="0.2">
+      <c r="E2" s="245"/>
+      <c r="F2" s="245"/>
+      <c r="G2" s="245"/>
+      <c r="H2" s="245"/>
+      <c r="I2" s="245"/>
+      <c r="J2" s="245"/>
+      <c r="K2" s="245"/>
+      <c r="L2" s="245"/>
+      <c r="M2" s="245"/>
+      <c r="N2" s="245"/>
+      <c r="O2" s="245"/>
+      <c r="P2" s="245"/>
+      <c r="Q2" s="245"/>
+      <c r="R2" s="245"/>
+      <c r="S2" s="245"/>
+      <c r="T2" s="245"/>
+      <c r="U2" s="245"/>
+      <c r="V2" s="245"/>
+      <c r="W2" s="245"/>
+      <c r="X2" s="245"/>
+      <c r="Y2" s="245"/>
+      <c r="Z2" s="245"/>
+    </row>
+    <row r="4" spans="1:28" s="10" customFormat="1" ht="126" x14ac:dyDescent="0.25">
       <c r="A4" s="9" t="s">
         <v>8</v>
       </c>
@@ -3405,14 +3405,14 @@
         <v>131</v>
       </c>
     </row>
-    <row r="5" spans="1:28" x14ac:dyDescent="0.2">
-      <c r="A5" s="285">
+    <row r="5" spans="1:28" x14ac:dyDescent="0.25">
+      <c r="A5" s="246">
         <v>46063</v>
       </c>
-      <c r="B5" s="286">
+      <c r="B5" s="249">
         <v>5</v>
       </c>
-      <c r="C5" s="287" t="s">
+      <c r="C5" s="252" t="s">
         <v>140</v>
       </c>
       <c r="D5" s="177">
@@ -3503,14 +3503,14 @@
         <f>Aerodinamika!G27</f>
         <v>1.3179692000000001</v>
       </c>
-      <c r="AB5" s="242" t="s">
+      <c r="AB5" s="243" t="s">
         <v>139</v>
       </c>
     </row>
-    <row r="6" spans="1:28" x14ac:dyDescent="0.2">
-      <c r="A6" s="288"/>
-      <c r="B6" s="289"/>
-      <c r="C6" s="290"/>
+    <row r="6" spans="1:28" x14ac:dyDescent="0.25">
+      <c r="A6" s="247"/>
+      <c r="B6" s="250"/>
+      <c r="C6" s="253"/>
       <c r="D6" s="177">
         <v>16</v>
       </c>
@@ -3595,12 +3595,12 @@
         <f>O5*X6</f>
         <v>0.79775867584824989</v>
       </c>
-      <c r="AB6" s="243"/>
-    </row>
-    <row r="7" spans="1:28" x14ac:dyDescent="0.2">
-      <c r="A7" s="288"/>
-      <c r="B7" s="289"/>
-      <c r="C7" s="290"/>
+      <c r="AB6" s="244"/>
+    </row>
+    <row r="7" spans="1:28" x14ac:dyDescent="0.25">
+      <c r="A7" s="247"/>
+      <c r="B7" s="250"/>
+      <c r="C7" s="253"/>
       <c r="D7" s="200">
         <v>31</v>
       </c>
@@ -3650,10 +3650,10 @@
       <c r="R7" s="176"/>
       <c r="S7" s="176"/>
     </row>
-    <row r="8" spans="1:28" x14ac:dyDescent="0.2">
-      <c r="A8" s="288"/>
-      <c r="B8" s="289"/>
-      <c r="C8" s="290"/>
+    <row r="8" spans="1:28" x14ac:dyDescent="0.25">
+      <c r="A8" s="247"/>
+      <c r="B8" s="250"/>
+      <c r="C8" s="253"/>
       <c r="D8" s="177">
         <v>60</v>
       </c>
@@ -3707,10 +3707,10 @@
         <v>132</v>
       </c>
     </row>
-    <row r="9" spans="1:28" x14ac:dyDescent="0.2">
-      <c r="A9" s="288"/>
-      <c r="B9" s="289"/>
-      <c r="C9" s="290"/>
+    <row r="9" spans="1:28" x14ac:dyDescent="0.25">
+      <c r="A9" s="247"/>
+      <c r="B9" s="250"/>
+      <c r="C9" s="253"/>
       <c r="D9" s="177">
         <v>89</v>
       </c>
@@ -3753,10 +3753,10 @@
         <v>10.243570073538624</v>
       </c>
     </row>
-    <row r="10" spans="1:28" x14ac:dyDescent="0.2">
-      <c r="A10" s="288"/>
-      <c r="B10" s="289"/>
-      <c r="C10" s="290"/>
+    <row r="10" spans="1:28" x14ac:dyDescent="0.25">
+      <c r="A10" s="247"/>
+      <c r="B10" s="250"/>
+      <c r="C10" s="253"/>
       <c r="D10" s="177">
         <v>104</v>
       </c>
@@ -3799,10 +3799,10 @@
         <v>10.180917681079487</v>
       </c>
     </row>
-    <row r="11" spans="1:28" x14ac:dyDescent="0.2">
-      <c r="A11" s="291"/>
-      <c r="B11" s="292"/>
-      <c r="C11" s="293"/>
+    <row r="11" spans="1:28" x14ac:dyDescent="0.25">
+      <c r="A11" s="248"/>
+      <c r="B11" s="251"/>
+      <c r="C11" s="254"/>
       <c r="D11" s="177">
         <v>115</v>
       </c>
@@ -3845,7 +3845,7 @@
         <v>9.796592606281104</v>
       </c>
     </row>
-    <row r="12" spans="1:28" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A12" s="206"/>
       <c r="B12" s="206"/>
       <c r="C12" s="206"/>
@@ -3867,24 +3867,24 @@
         <v>134</v>
       </c>
     </row>
-    <row r="13" spans="1:28" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:28" x14ac:dyDescent="0.25">
       <c r="D13" s="200" t="s">
         <v>135</v>
       </c>
-      <c r="E13" s="247" t="s">
+      <c r="E13" s="255" t="s">
         <v>136</v>
       </c>
-      <c r="F13" s="248"/>
-      <c r="G13" s="248"/>
-      <c r="H13" s="248"/>
-      <c r="I13" s="248"/>
-      <c r="J13" s="248"/>
-      <c r="K13" s="248"/>
-      <c r="L13" s="248"/>
-      <c r="M13" s="248"/>
-      <c r="N13" s="249"/>
-    </row>
-    <row r="14" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="F13" s="256"/>
+      <c r="G13" s="256"/>
+      <c r="H13" s="256"/>
+      <c r="I13" s="256"/>
+      <c r="J13" s="256"/>
+      <c r="K13" s="256"/>
+      <c r="L13" s="256"/>
+      <c r="M13" s="256"/>
+      <c r="N13" s="257"/>
+    </row>
+    <row r="14" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A14" s="206"/>
       <c r="B14" s="206"/>
       <c r="C14" s="206"/>
@@ -3893,7 +3893,7 @@
       <c r="G14" s="211"/>
       <c r="N14" s="212"/>
     </row>
-    <row r="15" spans="1:28" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A15" s="213"/>
       <c r="B15" s="213"/>
       <c r="C15" s="213"/>
@@ -3905,7 +3905,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="16" spans="1:28" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A16" s="206"/>
       <c r="B16" s="206"/>
       <c r="C16" s="206"/>
@@ -3913,37 +3913,37 @@
       <c r="F16" s="37"/>
       <c r="N16" s="212"/>
     </row>
-    <row r="17" spans="1:28" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A17" s="206"/>
       <c r="B17" s="206"/>
       <c r="C17" s="206"/>
-      <c r="D17" s="250" t="s">
+      <c r="D17" s="258" t="s">
         <v>138</v>
       </c>
-      <c r="E17" s="244"/>
-      <c r="F17" s="244"/>
-      <c r="G17" s="244"/>
-      <c r="H17" s="244"/>
-      <c r="I17" s="244"/>
-      <c r="J17" s="244"/>
-      <c r="K17" s="244"/>
-      <c r="L17" s="244"/>
-      <c r="M17" s="244"/>
-      <c r="N17" s="244"/>
-      <c r="O17" s="244"/>
-      <c r="P17" s="244"/>
-      <c r="Q17" s="244"/>
-      <c r="R17" s="244"/>
-      <c r="S17" s="244"/>
-      <c r="T17" s="244"/>
-      <c r="U17" s="244"/>
-      <c r="V17" s="244"/>
-      <c r="W17" s="244"/>
-      <c r="X17" s="244"/>
-      <c r="Y17" s="244"/>
-      <c r="Z17" s="244"/>
-    </row>
-    <row r="18" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="E17" s="245"/>
+      <c r="F17" s="245"/>
+      <c r="G17" s="245"/>
+      <c r="H17" s="245"/>
+      <c r="I17" s="245"/>
+      <c r="J17" s="245"/>
+      <c r="K17" s="245"/>
+      <c r="L17" s="245"/>
+      <c r="M17" s="245"/>
+      <c r="N17" s="245"/>
+      <c r="O17" s="245"/>
+      <c r="P17" s="245"/>
+      <c r="Q17" s="245"/>
+      <c r="R17" s="245"/>
+      <c r="S17" s="245"/>
+      <c r="T17" s="245"/>
+      <c r="U17" s="245"/>
+      <c r="V17" s="245"/>
+      <c r="W17" s="245"/>
+      <c r="X17" s="245"/>
+      <c r="Y17" s="245"/>
+      <c r="Z17" s="245"/>
+    </row>
+    <row r="18" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A18" s="206"/>
       <c r="B18" s="206"/>
       <c r="C18" s="206"/>
@@ -3960,7 +3960,7 @@
       <c r="N18" s="216"/>
       <c r="O18" s="214"/>
     </row>
-    <row r="19" spans="1:28" s="10" customFormat="1" ht="150" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:28" s="10" customFormat="1" ht="126" x14ac:dyDescent="0.25">
       <c r="A19" s="9" t="s">
         <v>8</v>
       </c>
@@ -4046,10 +4046,10 @@
         <v>131</v>
       </c>
     </row>
-    <row r="20" spans="1:28" ht="16.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="251"/>
-      <c r="B20" s="251"/>
-      <c r="C20" s="251"/>
+    <row r="20" spans="1:28" ht="16" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A20" s="259"/>
+      <c r="B20" s="259"/>
+      <c r="C20" s="259"/>
       <c r="D20" s="177">
         <v>3</v>
       </c>
@@ -4126,12 +4126,12 @@
       <c r="AA20" s="219">
         <v>1.35</v>
       </c>
-      <c r="AB20" s="242"/>
-    </row>
-    <row r="21" spans="1:28" x14ac:dyDescent="0.2">
-      <c r="A21" s="245"/>
-      <c r="B21" s="245"/>
-      <c r="C21" s="245"/>
+      <c r="AB20" s="243"/>
+    </row>
+    <row r="21" spans="1:28" x14ac:dyDescent="0.25">
+      <c r="A21" s="260"/>
+      <c r="B21" s="260"/>
+      <c r="C21" s="260"/>
       <c r="D21" s="177">
         <v>15</v>
       </c>
@@ -4202,12 +4202,12 @@
         <f>O20*X21</f>
         <v>1.0671545706141219</v>
       </c>
-      <c r="AB21" s="243"/>
-    </row>
-    <row r="22" spans="1:28" x14ac:dyDescent="0.2">
-      <c r="A22" s="245"/>
-      <c r="B22" s="245"/>
-      <c r="C22" s="245"/>
+      <c r="AB21" s="244"/>
+    </row>
+    <row r="22" spans="1:28" x14ac:dyDescent="0.25">
+      <c r="A22" s="260"/>
+      <c r="B22" s="260"/>
+      <c r="C22" s="260"/>
       <c r="D22" s="200">
         <v>27</v>
       </c>
@@ -4245,10 +4245,10 @@
       <c r="R22" s="176"/>
       <c r="S22" s="176"/>
     </row>
-    <row r="23" spans="1:28" x14ac:dyDescent="0.2">
-      <c r="A23" s="245"/>
-      <c r="B23" s="245"/>
-      <c r="C23" s="245"/>
+    <row r="23" spans="1:28" x14ac:dyDescent="0.25">
+      <c r="A23" s="260"/>
+      <c r="B23" s="260"/>
+      <c r="C23" s="260"/>
       <c r="D23" s="177">
         <v>4</v>
       </c>
@@ -4290,10 +4290,10 @@
         <v>132</v>
       </c>
     </row>
-    <row r="24" spans="1:28" x14ac:dyDescent="0.2">
-      <c r="A24" s="245"/>
-      <c r="B24" s="245"/>
-      <c r="C24" s="245"/>
+    <row r="24" spans="1:28" x14ac:dyDescent="0.25">
+      <c r="A24" s="260"/>
+      <c r="B24" s="260"/>
+      <c r="C24" s="260"/>
       <c r="D24" s="177">
         <v>5</v>
       </c>
@@ -4324,10 +4324,10 @@
         <v>11.973560791885415</v>
       </c>
     </row>
-    <row r="25" spans="1:28" x14ac:dyDescent="0.2">
-      <c r="A25" s="245"/>
-      <c r="B25" s="245"/>
-      <c r="C25" s="245"/>
+    <row r="25" spans="1:28" x14ac:dyDescent="0.25">
+      <c r="A25" s="260"/>
+      <c r="B25" s="260"/>
+      <c r="C25" s="260"/>
       <c r="D25" s="177">
         <v>6</v>
       </c>
@@ -4358,10 +4358,10 @@
         <v>12.445937737064785</v>
       </c>
     </row>
-    <row r="26" spans="1:28" x14ac:dyDescent="0.2">
-      <c r="A26" s="246"/>
-      <c r="B26" s="246"/>
-      <c r="C26" s="246"/>
+    <row r="26" spans="1:28" x14ac:dyDescent="0.25">
+      <c r="A26" s="261"/>
+      <c r="B26" s="261"/>
+      <c r="C26" s="261"/>
       <c r="D26" s="177">
         <v>7</v>
       </c>
@@ -4393,7 +4393,7 @@
       </c>
     </row>
   </sheetData>
-  <sheetProtection algorithmName="SHA-512" hashValue="YnNuFyjIZWP4o8siiNLOxJuXYMQvqdvZ9OrGGKpnMs1jyahS3pGpSVhE713S/7NZQvFDz0ZfCGMwTjhjC08CdQ==" saltValue="gCAgvRWICbIOkCsyhMCWFQ==" spinCount="100000" sheet="1" formatCells="0" formatColumns="0" formatRows="0"/>
+  <sheetProtection formatCells="0" formatColumns="0" formatRows="0"/>
   <mergeCells count="11">
     <mergeCell ref="AB20:AB21"/>
     <mergeCell ref="D2:Z2"/>
@@ -4414,21 +4414,21 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B782CE6F-4AAF-42E1-A4E9-B039A4011BD6}">
   <dimension ref="A1:L26"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="13" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="12.42578125" style="38" customWidth="1"/>
-    <col min="2" max="2" width="8.42578125" style="38" customWidth="1"/>
-    <col min="3" max="4" width="9.140625" style="38"/>
-    <col min="5" max="5" width="10.7109375" style="38" customWidth="1"/>
-    <col min="6" max="6" width="9.140625" style="38"/>
-    <col min="7" max="7" width="11.28515625" style="38" customWidth="1"/>
-    <col min="8" max="8" width="12.28515625" style="38" customWidth="1"/>
-    <col min="9" max="9" width="10.85546875" style="38" customWidth="1"/>
-    <col min="10" max="10" width="10.5703125" style="38" customWidth="1"/>
-    <col min="11" max="16384" width="9.140625" style="38"/>
+    <col min="1" max="1" width="12.453125" style="38" customWidth="1"/>
+    <col min="2" max="2" width="8.453125" style="38" customWidth="1"/>
+    <col min="3" max="4" width="9.1796875" style="38"/>
+    <col min="5" max="5" width="10.7265625" style="38" customWidth="1"/>
+    <col min="6" max="6" width="9.1796875" style="38"/>
+    <col min="7" max="7" width="11.26953125" style="38" customWidth="1"/>
+    <col min="8" max="8" width="12.26953125" style="38" customWidth="1"/>
+    <col min="9" max="9" width="10.81640625" style="38" customWidth="1"/>
+    <col min="10" max="10" width="10.54296875" style="38" customWidth="1"/>
+    <col min="11" max="16384" width="9.1796875" style="38"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" ht="15.75" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:12" ht="15" x14ac:dyDescent="0.3">
       <c r="A1" s="37"/>
       <c r="B1" s="10"/>
       <c r="C1" s="10"/>
@@ -4439,7 +4439,7 @@
       <c r="H1" s="10"/>
       <c r="I1" s="10"/>
     </row>
-    <row r="2" spans="1:12" ht="15.75" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:12" ht="15" x14ac:dyDescent="0.3">
       <c r="A2" s="39"/>
       <c r="B2" s="10"/>
       <c r="C2" s="10"/>
@@ -4450,21 +4450,21 @@
       <c r="H2" s="10"/>
       <c r="I2" s="10"/>
     </row>
-    <row r="3" spans="1:12" ht="23.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="252" t="s">
+    <row r="3" spans="1:12" ht="23.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="262" t="s">
         <v>107</v>
       </c>
-      <c r="B3" s="252"/>
-      <c r="C3" s="252"/>
-      <c r="D3" s="252"/>
-      <c r="E3" s="252"/>
-      <c r="F3" s="252"/>
-      <c r="G3" s="252"/>
-      <c r="H3" s="252"/>
-      <c r="I3" s="252"/>
-      <c r="J3" s="252"/>
-    </row>
-    <row r="4" spans="1:12" ht="15" x14ac:dyDescent="0.2">
+      <c r="B3" s="262"/>
+      <c r="C3" s="262"/>
+      <c r="D3" s="262"/>
+      <c r="E3" s="262"/>
+      <c r="F3" s="262"/>
+      <c r="G3" s="262"/>
+      <c r="H3" s="262"/>
+      <c r="I3" s="262"/>
+      <c r="J3" s="262"/>
+    </row>
+    <row r="4" spans="1:12" ht="14" x14ac:dyDescent="0.3">
       <c r="A4" s="10"/>
       <c r="B4" s="10"/>
       <c r="C4" s="10"/>
@@ -4475,7 +4475,7 @@
       <c r="H4" s="10"/>
       <c r="I4" s="10"/>
     </row>
-    <row r="5" spans="1:12" ht="90" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:12" ht="84" x14ac:dyDescent="0.3">
       <c r="A5" s="9"/>
       <c r="B5" s="9" t="s">
         <v>33</v>
@@ -4511,7 +4511,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="6" spans="1:12" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:12" ht="17.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="40"/>
       <c r="B6" s="9"/>
       <c r="C6" s="9"/>
@@ -4525,7 +4525,7 @@
       <c r="K6" s="45"/>
       <c r="L6" s="45"/>
     </row>
-    <row r="7" spans="1:12" ht="33" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:12" ht="33" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="40" t="s">
         <v>21</v>
       </c>
@@ -4566,7 +4566,7 @@
       </c>
       <c r="L7" s="45"/>
     </row>
-    <row r="8" spans="1:12" ht="15.75" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:12" ht="15" x14ac:dyDescent="0.3">
       <c r="A8" s="13"/>
       <c r="B8" s="97"/>
       <c r="C8" s="98"/>
@@ -4580,7 +4580,7 @@
       <c r="K8" s="45"/>
       <c r="L8" s="45"/>
     </row>
-    <row r="9" spans="1:12" ht="15.75" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:12" ht="15" x14ac:dyDescent="0.3">
       <c r="A9" s="13"/>
       <c r="B9" s="97"/>
       <c r="C9" s="98"/>
@@ -4594,7 +4594,7 @@
       <c r="K9" s="45"/>
       <c r="L9" s="45"/>
     </row>
-    <row r="10" spans="1:12" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:12" ht="42.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="102"/>
       <c r="B10" s="97"/>
       <c r="C10" s="13"/>
@@ -4608,62 +4608,62 @@
       <c r="K10" s="45"/>
       <c r="L10" s="45"/>
     </row>
-    <row r="11" spans="1:12" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H11" s="253" t="s">
+    <row r="11" spans="1:12" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="H11" s="263" t="s">
         <v>26</v>
       </c>
-      <c r="I11" s="256" t="s">
+      <c r="I11" s="266" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="12" spans="1:12" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H12" s="254"/>
-      <c r="I12" s="257"/>
-    </row>
-    <row r="13" spans="1:12" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H13" s="254"/>
-      <c r="I13" s="257"/>
-    </row>
-    <row r="14" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="H14" s="254"/>
-      <c r="I14" s="257"/>
-    </row>
-    <row r="15" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="H15" s="254"/>
-      <c r="I15" s="257"/>
-    </row>
-    <row r="16" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="H16" s="254"/>
-      <c r="I16" s="257"/>
-    </row>
-    <row r="17" spans="8:9" x14ac:dyDescent="0.2">
-      <c r="H17" s="254"/>
-      <c r="I17" s="257"/>
-    </row>
-    <row r="18" spans="8:9" x14ac:dyDescent="0.2">
-      <c r="H18" s="255"/>
-      <c r="I18" s="257"/>
-    </row>
-    <row r="19" spans="8:9" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="I19" s="257"/>
-    </row>
-    <row r="20" spans="8:9" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="I20" s="258"/>
-    </row>
-    <row r="21" spans="8:9" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:12" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="H12" s="264"/>
+      <c r="I12" s="267"/>
+    </row>
+    <row r="13" spans="1:12" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="H13" s="264"/>
+      <c r="I13" s="267"/>
+    </row>
+    <row r="14" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="H14" s="264"/>
+      <c r="I14" s="267"/>
+    </row>
+    <row r="15" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="H15" s="264"/>
+      <c r="I15" s="267"/>
+    </row>
+    <row r="16" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="H16" s="264"/>
+      <c r="I16" s="267"/>
+    </row>
+    <row r="17" spans="8:9" x14ac:dyDescent="0.3">
+      <c r="H17" s="264"/>
+      <c r="I17" s="267"/>
+    </row>
+    <row r="18" spans="8:9" x14ac:dyDescent="0.3">
+      <c r="H18" s="265"/>
+      <c r="I18" s="267"/>
+    </row>
+    <row r="19" spans="8:9" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="I19" s="267"/>
+    </row>
+    <row r="20" spans="8:9" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="I20" s="268"/>
+    </row>
+    <row r="21" spans="8:9" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="I21" s="57"/>
     </row>
-    <row r="22" spans="8:9" ht="12.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="23" spans="8:9" ht="15" x14ac:dyDescent="0.2">
+    <row r="22" spans="8:9" ht="12.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="23" spans="8:9" ht="14" x14ac:dyDescent="0.3">
       <c r="I23" s="56"/>
     </row>
-    <row r="24" spans="8:9" ht="15" x14ac:dyDescent="0.2">
+    <row r="24" spans="8:9" ht="14" x14ac:dyDescent="0.3">
       <c r="I24" s="56"/>
     </row>
-    <row r="25" spans="8:9" ht="15" x14ac:dyDescent="0.2">
+    <row r="25" spans="8:9" ht="14" x14ac:dyDescent="0.3">
       <c r="I25" s="56"/>
     </row>
-    <row r="26" spans="8:9" ht="15" x14ac:dyDescent="0.2">
+    <row r="26" spans="8:9" ht="14" x14ac:dyDescent="0.3">
       <c r="I26" s="56"/>
     </row>
   </sheetData>
@@ -4683,64 +4683,64 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:V77"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="14" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="2" width="13.28515625" style="14" customWidth="1"/>
-    <col min="3" max="3" width="26.140625" style="14" customWidth="1"/>
-    <col min="4" max="4" width="11.140625" style="14" customWidth="1"/>
-    <col min="5" max="5" width="12.140625" style="14" customWidth="1"/>
-    <col min="6" max="6" width="13.7109375" style="14" customWidth="1"/>
-    <col min="7" max="7" width="10.85546875" style="14" customWidth="1"/>
-    <col min="8" max="8" width="9.85546875" style="14" customWidth="1"/>
-    <col min="9" max="9" width="8.85546875" style="14" customWidth="1"/>
-    <col min="10" max="10" width="10.5703125" style="14" customWidth="1"/>
-    <col min="11" max="11" width="10.42578125" style="14" customWidth="1"/>
-    <col min="12" max="12" width="11.85546875" style="14" customWidth="1"/>
-    <col min="13" max="13" width="9.85546875" style="14" customWidth="1"/>
-    <col min="14" max="14" width="11.85546875" style="14" customWidth="1"/>
-    <col min="15" max="15" width="12.85546875" style="14" customWidth="1"/>
-    <col min="16" max="16" width="6.5703125" style="14" customWidth="1"/>
-    <col min="17" max="17" width="7.7109375" style="14" customWidth="1"/>
-    <col min="18" max="18" width="17.5703125" style="14" customWidth="1"/>
-    <col min="19" max="19" width="14.85546875" style="14" customWidth="1"/>
-    <col min="20" max="20" width="10.42578125" style="14" customWidth="1"/>
-    <col min="21" max="21" width="11.140625" style="14" customWidth="1"/>
-    <col min="22" max="22" width="13.42578125" style="14" customWidth="1"/>
-    <col min="23" max="16384" width="9.140625" style="14"/>
+    <col min="1" max="2" width="13.26953125" style="14" customWidth="1"/>
+    <col min="3" max="3" width="26.1796875" style="14" customWidth="1"/>
+    <col min="4" max="4" width="11.1796875" style="14" customWidth="1"/>
+    <col min="5" max="5" width="12.1796875" style="14" customWidth="1"/>
+    <col min="6" max="6" width="13.7265625" style="14" customWidth="1"/>
+    <col min="7" max="7" width="10.81640625" style="14" customWidth="1"/>
+    <col min="8" max="8" width="9.81640625" style="14" customWidth="1"/>
+    <col min="9" max="9" width="8.81640625" style="14" customWidth="1"/>
+    <col min="10" max="10" width="10.54296875" style="14" customWidth="1"/>
+    <col min="11" max="11" width="10.453125" style="14" customWidth="1"/>
+    <col min="12" max="12" width="11.81640625" style="14" customWidth="1"/>
+    <col min="13" max="13" width="9.81640625" style="14" customWidth="1"/>
+    <col min="14" max="14" width="11.81640625" style="14" customWidth="1"/>
+    <col min="15" max="15" width="12.81640625" style="14" customWidth="1"/>
+    <col min="16" max="16" width="6.54296875" style="14" customWidth="1"/>
+    <col min="17" max="17" width="7.7265625" style="14" customWidth="1"/>
+    <col min="18" max="18" width="17.54296875" style="14" customWidth="1"/>
+    <col min="19" max="19" width="14.81640625" style="14" customWidth="1"/>
+    <col min="20" max="20" width="10.453125" style="14" customWidth="1"/>
+    <col min="21" max="21" width="11.1796875" style="14" customWidth="1"/>
+    <col min="22" max="22" width="13.453125" style="14" customWidth="1"/>
+    <col min="23" max="16384" width="9.1796875" style="14"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:22" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C1" s="264" t="s">
+    <row r="1" spans="1:22" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C1" s="274" t="s">
         <v>14</v>
       </c>
-      <c r="D1" s="264"/>
+      <c r="D1" s="274"/>
       <c r="E1" s="15"/>
       <c r="S1" s="16"/>
     </row>
-    <row r="2" spans="1:22" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="265" t="s">
+    <row r="2" spans="1:22" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="275" t="s">
         <v>97</v>
       </c>
-      <c r="B2" s="265"/>
-      <c r="C2" s="265"/>
-      <c r="D2" s="265"/>
-      <c r="E2" s="265"/>
-      <c r="F2" s="265"/>
-      <c r="G2" s="265"/>
-      <c r="H2" s="265"/>
-      <c r="I2" s="265"/>
-      <c r="J2" s="265"/>
-      <c r="K2" s="265"/>
-      <c r="L2" s="265"/>
-      <c r="M2" s="265"/>
-      <c r="N2" s="265"/>
-      <c r="O2" s="265"/>
-      <c r="P2" s="265"/>
-      <c r="Q2" s="265"/>
-      <c r="R2" s="265"/>
-      <c r="S2" s="265"/>
-    </row>
-    <row r="3" spans="1:22" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B2" s="275"/>
+      <c r="C2" s="275"/>
+      <c r="D2" s="275"/>
+      <c r="E2" s="275"/>
+      <c r="F2" s="275"/>
+      <c r="G2" s="275"/>
+      <c r="H2" s="275"/>
+      <c r="I2" s="275"/>
+      <c r="J2" s="275"/>
+      <c r="K2" s="275"/>
+      <c r="L2" s="275"/>
+      <c r="M2" s="275"/>
+      <c r="N2" s="275"/>
+      <c r="O2" s="275"/>
+      <c r="P2" s="275"/>
+      <c r="Q2" s="275"/>
+      <c r="R2" s="275"/>
+      <c r="S2" s="275"/>
+    </row>
+    <row r="3" spans="1:22" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="17"/>
       <c r="B3" s="17"/>
       <c r="C3" s="18"/>
@@ -4761,10 +4761,10 @@
       <c r="R3" s="18"/>
       <c r="S3" s="18"/>
     </row>
-    <row r="4" spans="1:22" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:22" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="T4" s="26"/>
     </row>
-    <row r="5" spans="1:22" ht="100.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:22" ht="100.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="11" t="s">
         <v>8</v>
       </c>
@@ -4832,7 +4832,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="6" spans="1:22" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:22" ht="15" x14ac:dyDescent="0.3">
       <c r="A6" s="83">
         <f>Greitis!A5</f>
         <v>46063</v>
@@ -4840,7 +4840,7 @@
       <c r="B6" s="229" t="s">
         <v>141</v>
       </c>
-      <c r="C6" s="260" t="str">
+      <c r="C6" s="270" t="str">
         <f>Greitis!C5</f>
         <v>UAB ,,Ekopartneris", L. Ivinskio g. 65, Kaunas. Katilinė. Taršos šaltinis  Nr. 001.</v>
       </c>
@@ -4909,10 +4909,10 @@
         <v>63.1</v>
       </c>
     </row>
-    <row r="7" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A7" s="225"/>
       <c r="B7" s="226"/>
-      <c r="C7" s="261"/>
+      <c r="C7" s="271"/>
       <c r="D7" s="19"/>
       <c r="E7" s="20"/>
       <c r="F7" s="78">
@@ -4972,10 +4972,10 @@
         <v>62.7</v>
       </c>
     </row>
-    <row r="8" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A8" s="225"/>
       <c r="B8" s="226"/>
-      <c r="C8" s="261"/>
+      <c r="C8" s="271"/>
       <c r="D8" s="19"/>
       <c r="E8" s="20"/>
       <c r="F8" s="78">
@@ -5035,10 +5035,10 @@
         <v>63.3</v>
       </c>
     </row>
-    <row r="9" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A9" s="227"/>
       <c r="B9" s="227"/>
-      <c r="C9" s="261"/>
+      <c r="C9" s="271"/>
       <c r="D9" s="49"/>
       <c r="E9" s="49"/>
       <c r="F9" s="78">
@@ -5101,10 +5101,10 @@
         <v>63.033333333333339</v>
       </c>
     </row>
-    <row r="10" spans="1:22" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:22" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="227"/>
       <c r="B10" s="227"/>
-      <c r="C10" s="261"/>
+      <c r="C10" s="271"/>
       <c r="D10" s="49"/>
       <c r="E10" s="49"/>
       <c r="F10" s="78">
@@ -5154,20 +5154,20 @@
       </c>
       <c r="R10" s="49"/>
       <c r="S10" s="49"/>
-      <c r="T10" s="263" t="s">
+      <c r="T10" s="273" t="s">
         <v>28</v>
       </c>
-      <c r="U10" s="263" t="s">
+      <c r="U10" s="273" t="s">
         <v>29</v>
       </c>
-      <c r="V10" s="259" t="s">
+      <c r="V10" s="269" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="11" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A11" s="227"/>
       <c r="B11" s="227"/>
-      <c r="C11" s="261"/>
+      <c r="C11" s="271"/>
       <c r="D11" s="49"/>
       <c r="E11" s="49"/>
       <c r="F11" s="78">
@@ -5217,14 +5217,14 @@
       </c>
       <c r="R11" s="49"/>
       <c r="S11" s="49"/>
-      <c r="T11" s="263"/>
-      <c r="U11" s="263"/>
-      <c r="V11" s="259"/>
-    </row>
-    <row r="12" spans="1:22" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="T11" s="273"/>
+      <c r="U11" s="273"/>
+      <c r="V11" s="269"/>
+    </row>
+    <row r="12" spans="1:22" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="228"/>
       <c r="B12" s="228"/>
-      <c r="C12" s="262"/>
+      <c r="C12" s="272"/>
       <c r="D12" s="34"/>
       <c r="E12" s="34"/>
       <c r="F12" s="78">
@@ -5274,11 +5274,11 @@
       </c>
       <c r="R12" s="34"/>
       <c r="S12" s="34"/>
-      <c r="T12" s="263"/>
-      <c r="U12" s="263"/>
-      <c r="V12" s="259"/>
-    </row>
-    <row r="13" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="T12" s="273"/>
+      <c r="U12" s="273"/>
+      <c r="V12" s="269"/>
+    </row>
+    <row r="13" spans="1:22" x14ac:dyDescent="0.3">
       <c r="L13" s="81">
         <f>SUM(L6:L12)</f>
         <v>0.24000000000000002</v>
@@ -5292,7 +5292,7 @@
         <v>11.428571428571429</v>
       </c>
     </row>
-    <row r="14" spans="1:22" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:22" ht="30.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="L14" s="75" t="s">
         <v>25</v>
       </c>
@@ -5303,12 +5303,12 @@
         <v>145</v>
       </c>
     </row>
-    <row r="15" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A15" s="14" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="17" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A17" s="83">
         <f t="shared" ref="A17:F17" si="21">(A6)</f>
         <v>46063</v>
@@ -5317,7 +5317,7 @@
         <f t="shared" si="21"/>
         <v>3</v>
       </c>
-      <c r="C17" s="260" t="str">
+      <c r="C17" s="270" t="str">
         <f t="shared" si="21"/>
         <v>UAB ,,Ekopartneris", L. Ivinskio g. 65, Kaunas. Katilinė. Taršos šaltinis  Nr. 001.</v>
       </c>
@@ -5382,10 +5382,10 @@
         <v>105</v>
       </c>
     </row>
-    <row r="18" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A18" s="35"/>
       <c r="B18" s="32"/>
-      <c r="C18" s="261"/>
+      <c r="C18" s="271"/>
       <c r="D18" s="19"/>
       <c r="E18" s="20"/>
       <c r="F18" s="78">
@@ -5436,10 +5436,10 @@
       <c r="R18" s="23"/>
       <c r="S18" s="51"/>
     </row>
-    <row r="19" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A19" s="35"/>
       <c r="B19" s="32"/>
-      <c r="C19" s="261"/>
+      <c r="C19" s="271"/>
       <c r="D19" s="19"/>
       <c r="E19" s="20"/>
       <c r="F19" s="78">
@@ -5490,10 +5490,10 @@
       <c r="R19" s="23"/>
       <c r="S19" s="51"/>
     </row>
-    <row r="20" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A20" s="49"/>
       <c r="B20" s="49"/>
-      <c r="C20" s="261"/>
+      <c r="C20" s="271"/>
       <c r="D20" s="49"/>
       <c r="E20" s="49"/>
       <c r="F20" s="78">
@@ -5544,10 +5544,10 @@
       <c r="R20" s="49"/>
       <c r="S20" s="49"/>
     </row>
-    <row r="21" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A21" s="49"/>
       <c r="B21" s="49"/>
-      <c r="C21" s="261"/>
+      <c r="C21" s="271"/>
       <c r="D21" s="49"/>
       <c r="E21" s="49"/>
       <c r="F21" s="78">
@@ -5598,10 +5598,10 @@
       <c r="R21" s="49"/>
       <c r="S21" s="49"/>
     </row>
-    <row r="22" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A22" s="49"/>
       <c r="B22" s="49"/>
-      <c r="C22" s="261"/>
+      <c r="C22" s="271"/>
       <c r="D22" s="49"/>
       <c r="E22" s="49"/>
       <c r="F22" s="78">
@@ -5652,10 +5652,10 @@
       <c r="R22" s="49"/>
       <c r="S22" s="49"/>
     </row>
-    <row r="23" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A23" s="34"/>
       <c r="B23" s="34"/>
-      <c r="C23" s="262"/>
+      <c r="C23" s="272"/>
       <c r="D23" s="34"/>
       <c r="E23" s="34"/>
       <c r="F23" s="78">
@@ -5706,7 +5706,7 @@
       <c r="R23" s="34"/>
       <c r="S23" s="34"/>
     </row>
-    <row r="24" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:19" x14ac:dyDescent="0.3">
       <c r="L24" s="81">
         <f>SUM(L17:L23)</f>
         <v>0.23100000000000001</v>
@@ -5720,7 +5720,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="25" spans="1:19" ht="30" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:19" ht="28" x14ac:dyDescent="0.3">
       <c r="L25" s="75" t="s">
         <v>25</v>
       </c>
@@ -5731,14 +5731,14 @@
         <v>145</v>
       </c>
     </row>
-    <row r="26" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:19" x14ac:dyDescent="0.3">
       <c r="M26" s="113"/>
       <c r="N26" s="113"/>
       <c r="O26" s="113"/>
       <c r="P26" s="113"/>
       <c r="Q26" s="113"/>
     </row>
-    <row r="27" spans="1:19" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:19" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="L27" s="74"/>
       <c r="M27" s="153">
         <f>(M13+M24)</f>
@@ -5752,7 +5752,7 @@
       <c r="P27" s="113"/>
       <c r="Q27" s="113"/>
     </row>
-    <row r="28" spans="1:19" ht="48.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:19" ht="48.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="L28" s="74"/>
       <c r="M28" s="47" t="s">
         <v>96</v>
@@ -5761,20 +5761,20 @@
         <v>146</v>
       </c>
     </row>
-    <row r="37" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="74" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="37" ht="15" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="74" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A74" s="25"/>
       <c r="B74" s="25"/>
     </row>
-    <row r="75" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A75" s="25"/>
       <c r="B75" s="25"/>
     </row>
-    <row r="76" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A76" s="25"/>
       <c r="B76" s="25"/>
     </row>
-    <row r="77" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A77" s="25"/>
       <c r="B77" s="25"/>
     </row>
@@ -5805,54 +5805,54 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:Q30"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" outlineLevelCol="1" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="14" outlineLevelCol="1" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="11.28515625" style="14" customWidth="1"/>
-    <col min="2" max="2" width="13.28515625" style="14" customWidth="1"/>
-    <col min="3" max="3" width="20.85546875" style="14" customWidth="1"/>
-    <col min="4" max="4" width="12.7109375" style="14" customWidth="1"/>
-    <col min="5" max="6" width="16.140625" style="14" customWidth="1"/>
-    <col min="7" max="7" width="13.5703125" style="14" customWidth="1"/>
-    <col min="8" max="8" width="10.42578125" style="14" customWidth="1"/>
-    <col min="9" max="9" width="12.140625" style="14" customWidth="1" outlineLevel="1"/>
+    <col min="1" max="1" width="11.26953125" style="14" customWidth="1"/>
+    <col min="2" max="2" width="13.26953125" style="14" customWidth="1"/>
+    <col min="3" max="3" width="20.81640625" style="14" customWidth="1"/>
+    <col min="4" max="4" width="12.7265625" style="14" customWidth="1"/>
+    <col min="5" max="6" width="16.1796875" style="14" customWidth="1"/>
+    <col min="7" max="7" width="13.54296875" style="14" customWidth="1"/>
+    <col min="8" max="8" width="10.453125" style="14" customWidth="1"/>
+    <col min="9" max="9" width="12.1796875" style="14" customWidth="1" outlineLevel="1"/>
     <col min="10" max="10" width="10" style="14" customWidth="1" outlineLevel="1"/>
-    <col min="11" max="11" width="11.7109375" style="14" customWidth="1"/>
-    <col min="12" max="12" width="11.5703125" style="14" customWidth="1"/>
+    <col min="11" max="11" width="11.7265625" style="14" customWidth="1"/>
+    <col min="12" max="12" width="11.54296875" style="14" customWidth="1"/>
     <col min="13" max="13" width="17" style="14" customWidth="1"/>
-    <col min="14" max="14" width="15.28515625" style="14" customWidth="1"/>
-    <col min="15" max="16384" width="9.140625" style="14"/>
+    <col min="14" max="14" width="15.26953125" style="14" customWidth="1"/>
+    <col min="15" max="16384" width="9.1796875" style="14"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C1" s="264" t="s">
+    <row r="1" spans="1:17" ht="30.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C1" s="274" t="s">
         <v>15</v>
       </c>
-      <c r="D1" s="264"/>
+      <c r="D1" s="274"/>
       <c r="Q1" s="16"/>
     </row>
-    <row r="2" spans="1:17" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C2" s="266" t="s">
+    <row r="2" spans="1:17" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C2" s="276" t="s">
         <v>98</v>
       </c>
-      <c r="D2" s="266"/>
-      <c r="E2" s="266"/>
-      <c r="F2" s="266"/>
-      <c r="G2" s="266"/>
-      <c r="H2" s="266"/>
-      <c r="I2" s="266"/>
-      <c r="J2" s="266"/>
-      <c r="K2" s="266"/>
-      <c r="L2" s="266"/>
-      <c r="M2" s="266"/>
+      <c r="D2" s="276"/>
+      <c r="E2" s="276"/>
+      <c r="F2" s="276"/>
+      <c r="G2" s="276"/>
+      <c r="H2" s="276"/>
+      <c r="I2" s="276"/>
+      <c r="J2" s="276"/>
+      <c r="K2" s="276"/>
+      <c r="L2" s="276"/>
+      <c r="M2" s="276"/>
       <c r="Q2" s="16"/>
     </row>
-    <row r="3" spans="1:17" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:17" ht="12" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C3" s="24"/>
       <c r="H3" s="25"/>
       <c r="Q3" s="16"/>
     </row>
-    <row r="4" spans="1:17" ht="8.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="5" spans="1:17" ht="126.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:17" ht="8.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="5" spans="1:17" ht="126.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="117" t="s">
         <v>8</v>
       </c>
@@ -5896,7 +5896,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="6" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="87">
         <f>Paėmimas!A6</f>
         <v>46063</v>
@@ -5905,7 +5905,7 @@
         <f>Paėmimas!B6</f>
         <v>3</v>
       </c>
-      <c r="C6" s="260" t="str">
+      <c r="C6" s="270" t="str">
         <f>Paėmimas!C6</f>
         <v>UAB ,,Ekopartneris", L. Ivinskio g. 65, Kaunas. Katilinė. Taršos šaltinis  Nr. 001.</v>
       </c>
@@ -5954,10 +5954,10 @@
         <v>1 linija, 1 filtras</v>
       </c>
     </row>
-    <row r="7" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="59"/>
       <c r="B7" s="23"/>
-      <c r="C7" s="261"/>
+      <c r="C7" s="271"/>
       <c r="D7" s="58">
         <f>Paėmimas!L7</f>
         <v>3.5999999999999997E-2</v>
@@ -5991,10 +5991,10 @@
       <c r="M7" s="60"/>
       <c r="N7" s="32"/>
     </row>
-    <row r="8" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="59"/>
       <c r="B8" s="23"/>
-      <c r="C8" s="261"/>
+      <c r="C8" s="271"/>
       <c r="D8" s="58">
         <f>Paėmimas!L8</f>
         <v>3.5999999999999997E-2</v>
@@ -6028,10 +6028,10 @@
       <c r="M8" s="60"/>
       <c r="N8" s="32"/>
     </row>
-    <row r="9" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="59"/>
       <c r="B9" s="23"/>
-      <c r="C9" s="261"/>
+      <c r="C9" s="271"/>
       <c r="D9" s="58">
         <f>Paėmimas!L9</f>
         <v>3.5999999999999997E-2</v>
@@ -6065,10 +6065,10 @@
       <c r="M9" s="60"/>
       <c r="N9" s="32"/>
     </row>
-    <row r="10" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="59"/>
       <c r="B10" s="23"/>
-      <c r="C10" s="261"/>
+      <c r="C10" s="271"/>
       <c r="D10" s="58">
         <f>Paėmimas!L10</f>
         <v>3.5999999999999997E-2</v>
@@ -6102,10 +6102,10 @@
       <c r="M10" s="60"/>
       <c r="N10" s="32"/>
     </row>
-    <row r="11" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="59"/>
       <c r="B11" s="23"/>
-      <c r="C11" s="261"/>
+      <c r="C11" s="271"/>
       <c r="D11" s="58">
         <f>Paėmimas!L11</f>
         <v>3.3000000000000002E-2</v>
@@ -6139,10 +6139,10 @@
       <c r="M11" s="60"/>
       <c r="N11" s="32"/>
     </row>
-    <row r="12" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="61"/>
       <c r="B12" s="62"/>
-      <c r="C12" s="261"/>
+      <c r="C12" s="271"/>
       <c r="D12" s="58">
         <f>Paėmimas!L12</f>
         <v>0.03</v>
@@ -6176,7 +6176,7 @@
       <c r="M12" s="63"/>
       <c r="N12" s="22"/>
     </row>
-    <row r="13" spans="1:17" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:17" ht="17.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C13" s="94"/>
       <c r="D13" s="94"/>
       <c r="E13" s="94"/>
@@ -6192,7 +6192,7 @@
       </c>
       <c r="J13" s="94"/>
     </row>
-    <row r="14" spans="1:17" ht="34.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:17" ht="34.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C14" s="95"/>
       <c r="D14" s="95"/>
       <c r="E14" s="95"/>
@@ -6206,7 +6206,7 @@
       </c>
       <c r="J14" s="95"/>
     </row>
-    <row r="15" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C15" s="95"/>
       <c r="D15" s="95"/>
       <c r="E15" s="95"/>
@@ -6216,7 +6216,7 @@
       <c r="I15" s="95"/>
       <c r="J15" s="95"/>
     </row>
-    <row r="17" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A17" s="87">
         <f>Paėmimas!A17</f>
         <v>46063</v>
@@ -6225,7 +6225,7 @@
         <f>Paėmimas!B17</f>
         <v>3</v>
       </c>
-      <c r="C17" s="260" t="str">
+      <c r="C17" s="270" t="str">
         <f>Paėmimas!C17</f>
         <v>UAB ,,Ekopartneris", L. Ivinskio g. 65, Kaunas. Katilinė. Taršos šaltinis  Nr. 001.</v>
       </c>
@@ -6274,10 +6274,10 @@
         <v>2 linija, 1 filtras</v>
       </c>
     </row>
-    <row r="18" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A18" s="59"/>
       <c r="B18" s="23"/>
-      <c r="C18" s="261"/>
+      <c r="C18" s="271"/>
       <c r="D18" s="58">
         <f>Paėmimas!L18</f>
         <v>3.3000000000000002E-2</v>
@@ -6311,10 +6311,10 @@
       <c r="M18" s="60"/>
       <c r="N18" s="32"/>
     </row>
-    <row r="19" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A19" s="59"/>
       <c r="B19" s="23"/>
-      <c r="C19" s="261"/>
+      <c r="C19" s="271"/>
       <c r="D19" s="58">
         <f>Paėmimas!L19</f>
         <v>3.3000000000000002E-2</v>
@@ -6348,10 +6348,10 @@
       <c r="M19" s="60"/>
       <c r="N19" s="32"/>
     </row>
-    <row r="20" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A20" s="59"/>
       <c r="B20" s="23"/>
-      <c r="C20" s="261"/>
+      <c r="C20" s="271"/>
       <c r="D20" s="58">
         <f>Paėmimas!L20</f>
         <v>3.5999999999999997E-2</v>
@@ -6385,10 +6385,10 @@
       <c r="M20" s="60"/>
       <c r="N20" s="32"/>
     </row>
-    <row r="21" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A21" s="59"/>
       <c r="B21" s="23"/>
-      <c r="C21" s="261"/>
+      <c r="C21" s="271"/>
       <c r="D21" s="58">
         <f>Paėmimas!L21</f>
         <v>3.3000000000000002E-2</v>
@@ -6422,10 +6422,10 @@
       <c r="M21" s="60"/>
       <c r="N21" s="32"/>
     </row>
-    <row r="22" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A22" s="59"/>
       <c r="B22" s="23"/>
-      <c r="C22" s="261"/>
+      <c r="C22" s="271"/>
       <c r="D22" s="58">
         <f>Paėmimas!L22</f>
         <v>3.3000000000000002E-2</v>
@@ -6459,10 +6459,10 @@
       <c r="M22" s="60"/>
       <c r="N22" s="32"/>
     </row>
-    <row r="23" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A23" s="61"/>
       <c r="B23" s="62"/>
-      <c r="C23" s="261"/>
+      <c r="C23" s="271"/>
       <c r="D23" s="58">
         <f>Paėmimas!L23</f>
         <v>3.3000000000000002E-2</v>
@@ -6496,7 +6496,7 @@
       <c r="M23" s="63"/>
       <c r="N23" s="22"/>
     </row>
-    <row r="24" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:14" x14ac:dyDescent="0.3">
       <c r="C24" s="94"/>
       <c r="D24" s="94"/>
       <c r="E24" s="94"/>
@@ -6519,7 +6519,7 @@
         <v>1.047386335075599</v>
       </c>
     </row>
-    <row r="25" spans="1:14" ht="60" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:14" ht="56" x14ac:dyDescent="0.3">
       <c r="C25" s="95"/>
       <c r="D25" s="95"/>
       <c r="E25" s="95"/>
@@ -6538,7 +6538,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="26" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:14" x14ac:dyDescent="0.3">
       <c r="C26" s="96"/>
       <c r="D26" s="96"/>
       <c r="E26" s="96"/>
@@ -6548,7 +6548,7 @@
       <c r="I26" s="96"/>
       <c r="J26" s="96"/>
     </row>
-    <row r="27" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:14" x14ac:dyDescent="0.3">
       <c r="C27" s="96"/>
       <c r="D27" s="96"/>
       <c r="E27" s="96"/>
@@ -6564,7 +6564,7 @@
       </c>
       <c r="J27" s="96"/>
     </row>
-    <row r="28" spans="1:14" ht="55.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:14" ht="55.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C28" s="96"/>
       <c r="D28" s="96"/>
       <c r="E28" s="96"/>
@@ -6578,7 +6578,7 @@
       </c>
       <c r="J28" s="96"/>
     </row>
-    <row r="29" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:14" x14ac:dyDescent="0.3">
       <c r="C29" s="96"/>
       <c r="D29" s="96"/>
       <c r="E29" s="96"/>
@@ -6588,7 +6588,7 @@
       <c r="I29" s="96"/>
       <c r="J29" s="96"/>
     </row>
-    <row r="30" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:14" x14ac:dyDescent="0.3">
       <c r="C30" s="96"/>
       <c r="D30" s="96"/>
       <c r="E30" s="96"/>
@@ -6622,64 +6622,64 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:R8"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="14" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="11.7109375" style="14" customWidth="1"/>
-    <col min="2" max="2" width="13.42578125" style="14" customWidth="1"/>
-    <col min="3" max="3" width="24.5703125" style="14" customWidth="1"/>
-    <col min="4" max="4" width="8.140625" style="14" customWidth="1"/>
-    <col min="5" max="5" width="11.5703125" style="14" customWidth="1"/>
-    <col min="6" max="6" width="12.28515625" style="14" customWidth="1"/>
+    <col min="1" max="1" width="11.7265625" style="14" customWidth="1"/>
+    <col min="2" max="2" width="13.453125" style="14" customWidth="1"/>
+    <col min="3" max="3" width="24.54296875" style="14" customWidth="1"/>
+    <col min="4" max="4" width="8.1796875" style="14" customWidth="1"/>
+    <col min="5" max="5" width="11.54296875" style="14" customWidth="1"/>
+    <col min="6" max="6" width="12.26953125" style="14" customWidth="1"/>
     <col min="7" max="7" width="11" style="14" customWidth="1"/>
-    <col min="8" max="9" width="10.28515625" style="14" customWidth="1"/>
-    <col min="10" max="10" width="11.140625" style="14" customWidth="1"/>
-    <col min="11" max="11" width="14.28515625" style="14" customWidth="1"/>
-    <col min="12" max="12" width="11.28515625" style="14" customWidth="1"/>
-    <col min="13" max="13" width="10.5703125" style="14" customWidth="1"/>
-    <col min="14" max="14" width="17.7109375" style="14" customWidth="1"/>
-    <col min="15" max="15" width="8.28515625" style="14" customWidth="1"/>
-    <col min="16" max="16" width="17.140625" style="14" customWidth="1"/>
-    <col min="17" max="17" width="9.140625" style="14"/>
-    <col min="18" max="18" width="9.5703125" style="14" bestFit="1" customWidth="1"/>
-    <col min="19" max="16384" width="9.140625" style="14"/>
+    <col min="8" max="9" width="10.26953125" style="14" customWidth="1"/>
+    <col min="10" max="10" width="11.1796875" style="14" customWidth="1"/>
+    <col min="11" max="11" width="14.26953125" style="14" customWidth="1"/>
+    <col min="12" max="12" width="11.26953125" style="14" customWidth="1"/>
+    <col min="13" max="13" width="10.54296875" style="14" customWidth="1"/>
+    <col min="14" max="14" width="17.7265625" style="14" customWidth="1"/>
+    <col min="15" max="15" width="8.26953125" style="14" customWidth="1"/>
+    <col min="16" max="16" width="17.1796875" style="14" customWidth="1"/>
+    <col min="17" max="17" width="9.1796875" style="14"/>
+    <col min="18" max="18" width="9.54296875" style="14" bestFit="1" customWidth="1"/>
+    <col min="19" max="16384" width="9.1796875" style="14"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C1" s="264" t="s">
+    <row r="1" spans="1:18" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C1" s="274" t="s">
         <v>16</v>
       </c>
-      <c r="D1" s="264"/>
+      <c r="D1" s="274"/>
       <c r="R1" s="16"/>
     </row>
-    <row r="2" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A2" s="266" t="s">
+    <row r="2" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A2" s="276" t="s">
         <v>99</v>
       </c>
-      <c r="B2" s="266"/>
-      <c r="C2" s="266"/>
-      <c r="D2" s="266"/>
-      <c r="E2" s="266"/>
-      <c r="F2" s="266"/>
-      <c r="G2" s="266"/>
-      <c r="H2" s="266"/>
-      <c r="I2" s="266"/>
-      <c r="J2" s="266"/>
-      <c r="K2" s="266"/>
-      <c r="L2" s="266"/>
-      <c r="M2" s="266"/>
-      <c r="N2" s="266"/>
+      <c r="B2" s="276"/>
+      <c r="C2" s="276"/>
+      <c r="D2" s="276"/>
+      <c r="E2" s="276"/>
+      <c r="F2" s="276"/>
+      <c r="G2" s="276"/>
+      <c r="H2" s="276"/>
+      <c r="I2" s="276"/>
+      <c r="J2" s="276"/>
+      <c r="K2" s="276"/>
+      <c r="L2" s="276"/>
+      <c r="M2" s="276"/>
+      <c r="N2" s="276"/>
       <c r="O2" s="156"/>
     </row>
-    <row r="3" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:18" x14ac:dyDescent="0.3">
       <c r="F3" s="27"/>
       <c r="L3" s="16"/>
       <c r="M3" s="16"/>
     </row>
-    <row r="4" spans="1:18" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:18" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="L4" s="16"/>
       <c r="M4" s="16"/>
     </row>
-    <row r="5" spans="1:18" ht="88.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:18" ht="88.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="117" t="s">
         <v>8</v>
       </c>
@@ -6729,7 +6729,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="6" spans="1:18" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:18" ht="17.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="66">
         <f>Paėmimas!A6</f>
         <v>46063</v>
@@ -6738,7 +6738,7 @@
         <f>Svėrimas!A6</f>
         <v>3</v>
       </c>
-      <c r="C6" s="267" t="str">
+      <c r="C6" s="277" t="str">
         <f>Paėmimas!C6</f>
         <v>UAB ,,Ekopartneris", L. Ivinskio g. 65, Kaunas. Katilinė. Taršos šaltinis  Nr. 001.</v>
       </c>
@@ -6758,7 +6758,7 @@
         <f>Svėrimas!M9</f>
         <v>1.0000000000021103E-4</v>
       </c>
-      <c r="H6" s="284">
+      <c r="H6" s="242">
         <f>Svėrimas!M11/O6</f>
         <v>9.9999999996214228E-5</v>
       </c>
@@ -6794,10 +6794,10 @@
         <v>1 ir 2 linijos, 1 filtras</v>
       </c>
     </row>
-    <row r="7" spans="1:18" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:18" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="66"/>
       <c r="B7" s="67"/>
-      <c r="C7" s="267"/>
+      <c r="C7" s="277"/>
       <c r="D7" s="68"/>
       <c r="E7" s="127"/>
       <c r="F7" s="129"/>
@@ -6812,10 +6812,10 @@
       <c r="O7" s="32"/>
       <c r="P7" s="65"/>
     </row>
-    <row r="8" spans="1:18" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:18" ht="22.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="76"/>
       <c r="B8" s="65"/>
-      <c r="C8" s="268"/>
+      <c r="C8" s="278"/>
       <c r="D8" s="68"/>
       <c r="E8" s="127"/>
       <c r="F8" s="129"/>
@@ -6850,97 +6850,97 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{330ECBA1-822C-4C0F-89AB-CB2C7AD5643F}">
   <dimension ref="A1:P18"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="14" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="13.7109375" style="112" customWidth="1"/>
-    <col min="2" max="2" width="25.140625" style="112" customWidth="1"/>
-    <col min="3" max="3" width="7.42578125" style="112" customWidth="1"/>
-    <col min="4" max="4" width="12.85546875" style="112" customWidth="1"/>
-    <col min="5" max="5" width="11.140625" style="112" customWidth="1"/>
-    <col min="6" max="6" width="10.85546875" style="112" customWidth="1"/>
-    <col min="7" max="7" width="10.42578125" style="112" customWidth="1"/>
+    <col min="1" max="1" width="13.7265625" style="112" customWidth="1"/>
+    <col min="2" max="2" width="25.1796875" style="112" customWidth="1"/>
+    <col min="3" max="3" width="7.453125" style="112" customWidth="1"/>
+    <col min="4" max="4" width="12.81640625" style="112" customWidth="1"/>
+    <col min="5" max="5" width="11.1796875" style="112" customWidth="1"/>
+    <col min="6" max="6" width="10.81640625" style="112" customWidth="1"/>
+    <col min="7" max="7" width="10.453125" style="112" customWidth="1"/>
     <col min="8" max="8" width="18" style="112" customWidth="1"/>
-    <col min="9" max="9" width="11.28515625" style="112" customWidth="1"/>
-    <col min="10" max="10" width="10.85546875" style="112" customWidth="1"/>
+    <col min="9" max="9" width="11.26953125" style="112" customWidth="1"/>
+    <col min="10" max="10" width="10.81640625" style="112" customWidth="1"/>
     <col min="11" max="11" width="11" style="112" customWidth="1"/>
-    <col min="12" max="12" width="11.140625" style="112" customWidth="1"/>
-    <col min="13" max="13" width="20.42578125" style="112" customWidth="1"/>
-    <col min="14" max="14" width="16.85546875" style="112" customWidth="1"/>
-    <col min="15" max="15" width="31.140625" style="112" customWidth="1"/>
-    <col min="16" max="16384" width="9.140625" style="112"/>
+    <col min="12" max="12" width="11.1796875" style="112" customWidth="1"/>
+    <col min="13" max="13" width="20.453125" style="112" customWidth="1"/>
+    <col min="14" max="14" width="16.81640625" style="112" customWidth="1"/>
+    <col min="15" max="15" width="31.1796875" style="112" customWidth="1"/>
+    <col min="16" max="16384" width="9.1796875" style="112"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" ht="26.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="C1" s="264" t="s">
+    <row r="1" spans="1:16" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C1" s="274" t="s">
         <v>17</v>
       </c>
-      <c r="D1" s="264"/>
-      <c r="E1" s="264"/>
-      <c r="F1" s="264"/>
-    </row>
-    <row r="2" spans="1:16" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="266" t="s">
+      <c r="D1" s="274"/>
+      <c r="E1" s="274"/>
+      <c r="F1" s="274"/>
+    </row>
+    <row r="2" spans="1:16" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="276" t="s">
         <v>100</v>
       </c>
-      <c r="B2" s="266"/>
-      <c r="C2" s="266"/>
-      <c r="D2" s="266"/>
-      <c r="E2" s="266"/>
-      <c r="F2" s="266"/>
-      <c r="G2" s="266"/>
-      <c r="H2" s="266"/>
-      <c r="I2" s="266"/>
-      <c r="J2" s="266"/>
-      <c r="K2" s="266"/>
-      <c r="L2" s="266"/>
-      <c r="M2" s="266"/>
-      <c r="N2" s="266"/>
-      <c r="O2" s="266"/>
-    </row>
-    <row r="4" spans="1:16" ht="60" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="275" t="s">
+      <c r="B2" s="276"/>
+      <c r="C2" s="276"/>
+      <c r="D2" s="276"/>
+      <c r="E2" s="276"/>
+      <c r="F2" s="276"/>
+      <c r="G2" s="276"/>
+      <c r="H2" s="276"/>
+      <c r="I2" s="276"/>
+      <c r="J2" s="276"/>
+      <c r="K2" s="276"/>
+      <c r="L2" s="276"/>
+      <c r="M2" s="276"/>
+      <c r="N2" s="276"/>
+      <c r="O2" s="276"/>
+    </row>
+    <row r="4" spans="1:16" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="280" t="s">
         <v>80</v>
       </c>
-      <c r="B4" s="275" t="s">
+      <c r="B4" s="280" t="s">
         <v>9</v>
       </c>
-      <c r="C4" s="272" t="s">
+      <c r="C4" s="291" t="s">
         <v>81</v>
       </c>
-      <c r="D4" s="272" t="s">
+      <c r="D4" s="291" t="s">
         <v>82</v>
       </c>
-      <c r="E4" s="272" t="s">
+      <c r="E4" s="291" t="s">
         <v>83</v>
       </c>
-      <c r="F4" s="272"/>
-      <c r="G4" s="272"/>
-      <c r="H4" s="272" t="s">
+      <c r="F4" s="291"/>
+      <c r="G4" s="291"/>
+      <c r="H4" s="291" t="s">
         <v>13</v>
       </c>
-      <c r="I4" s="279" t="s">
+      <c r="I4" s="284" t="s">
         <v>84</v>
       </c>
-      <c r="J4" s="274" t="s">
+      <c r="J4" s="279" t="s">
         <v>85</v>
       </c>
-      <c r="K4" s="274"/>
-      <c r="L4" s="274"/>
-      <c r="M4" s="281" t="s">
+      <c r="K4" s="279"/>
+      <c r="L4" s="279"/>
+      <c r="M4" s="286" t="s">
         <v>86</v>
       </c>
-      <c r="N4" s="274" t="s">
+      <c r="N4" s="279" t="s">
         <v>13</v>
       </c>
-      <c r="O4" s="277" t="s">
+      <c r="O4" s="282" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="5" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="276"/>
-      <c r="B5" s="276"/>
-      <c r="C5" s="273"/>
-      <c r="D5" s="272"/>
+    <row r="5" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="281"/>
+      <c r="B5" s="281"/>
+      <c r="C5" s="292"/>
+      <c r="D5" s="291"/>
       <c r="E5" s="146">
         <v>1</v>
       </c>
@@ -6950,8 +6950,8 @@
       <c r="G5" s="146">
         <v>3</v>
       </c>
-      <c r="H5" s="272"/>
-      <c r="I5" s="280"/>
+      <c r="H5" s="291"/>
+      <c r="I5" s="285"/>
       <c r="J5" s="12">
         <v>1</v>
       </c>
@@ -6961,16 +6961,16 @@
       <c r="L5" s="12">
         <v>3</v>
       </c>
-      <c r="M5" s="282"/>
-      <c r="N5" s="274"/>
-      <c r="O5" s="278"/>
-    </row>
-    <row r="6" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="M5" s="287"/>
+      <c r="N5" s="279"/>
+      <c r="O5" s="283"/>
+    </row>
+    <row r="6" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="170" t="str">
         <f>Paėmimas!B6</f>
         <v>3</v>
       </c>
-      <c r="B6" s="269" t="str">
+      <c r="B6" s="288" t="str">
         <f>Paėmimas!C6</f>
         <v>UAB ,,Ekopartneris", L. Ivinskio g. 65, Kaunas. Katilinė. Taršos šaltinis  Nr. 001.</v>
       </c>
@@ -7017,9 +7017,9 @@
         <v>106</v>
       </c>
     </row>
-    <row r="7" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="32"/>
-      <c r="B7" s="270"/>
+      <c r="B7" s="289"/>
       <c r="C7" s="31"/>
       <c r="D7" s="28"/>
       <c r="E7" s="231"/>
@@ -7037,9 +7037,9 @@
       <c r="N7" s="30"/>
       <c r="O7" s="141"/>
     </row>
-    <row r="8" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="32"/>
-      <c r="B8" s="270"/>
+      <c r="B8" s="289"/>
       <c r="C8" s="31"/>
       <c r="D8" s="106"/>
       <c r="E8" s="231"/>
@@ -7057,9 +7057,9 @@
       <c r="N8" s="107"/>
       <c r="O8" s="142"/>
     </row>
-    <row r="9" spans="1:16" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:16" ht="17" x14ac:dyDescent="0.45">
       <c r="A9" s="32"/>
-      <c r="B9" s="270"/>
+      <c r="B9" s="289"/>
       <c r="C9" s="31">
         <v>2</v>
       </c>
@@ -7094,9 +7094,9 @@
       </c>
       <c r="P9" s="114"/>
     </row>
-    <row r="10" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A10" s="32"/>
-      <c r="B10" s="270"/>
+      <c r="B10" s="289"/>
       <c r="C10" s="31"/>
       <c r="D10" s="106"/>
       <c r="E10" s="231"/>
@@ -7111,9 +7111,9 @@
       <c r="N10" s="107"/>
       <c r="O10" s="147"/>
     </row>
-    <row r="11" spans="1:16" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:16" ht="17" x14ac:dyDescent="0.45">
       <c r="A11" s="32"/>
-      <c r="B11" s="270"/>
+      <c r="B11" s="289"/>
       <c r="C11" s="31">
         <v>41</v>
       </c>
@@ -7147,9 +7147,9 @@
         <v>88</v>
       </c>
     </row>
-    <row r="12" spans="1:16" ht="30.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:16" ht="30.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A12" s="32"/>
-      <c r="B12" s="270"/>
+      <c r="B12" s="289"/>
       <c r="C12" s="138" t="s">
         <v>41</v>
       </c>
@@ -7183,9 +7183,9 @@
         <v>89</v>
       </c>
     </row>
-    <row r="13" spans="1:16" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:16" ht="17" x14ac:dyDescent="0.45">
       <c r="A13" s="32"/>
-      <c r="B13" s="270"/>
+      <c r="B13" s="289"/>
       <c r="C13" s="139" t="s">
         <v>42</v>
       </c>
@@ -7219,9 +7219,9 @@
         <v>90</v>
       </c>
     </row>
-    <row r="14" spans="1:16" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:16" ht="17" x14ac:dyDescent="0.45">
       <c r="A14" s="32"/>
-      <c r="B14" s="270"/>
+      <c r="B14" s="289"/>
       <c r="C14" s="139" t="s">
         <v>43</v>
       </c>
@@ -7255,9 +7255,9 @@
         <v>91</v>
       </c>
     </row>
-    <row r="15" spans="1:16" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:16" ht="17" x14ac:dyDescent="0.45">
       <c r="A15" s="32"/>
-      <c r="B15" s="270"/>
+      <c r="B15" s="289"/>
       <c r="C15" s="140" t="s">
         <v>44</v>
       </c>
@@ -7291,9 +7291,9 @@
         <v>92</v>
       </c>
     </row>
-    <row r="16" spans="1:16" ht="32.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:16" ht="32.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A16" s="22"/>
-      <c r="B16" s="271"/>
+      <c r="B16" s="290"/>
       <c r="C16" s="31"/>
       <c r="D16" s="109"/>
       <c r="E16" s="21"/>
@@ -7313,10 +7313,10 @@
         <v>93</v>
       </c>
     </row>
-    <row r="17" spans="11:11" x14ac:dyDescent="0.2">
+    <row r="17" spans="11:11" x14ac:dyDescent="0.25">
       <c r="K17" s="113"/>
     </row>
-    <row r="18" spans="11:11" x14ac:dyDescent="0.2">
+    <row r="18" spans="11:11" x14ac:dyDescent="0.25">
       <c r="K18" s="113"/>
     </row>
   </sheetData>
@@ -7327,6 +7327,11 @@
     </sortState>
   </autoFilter>
   <mergeCells count="14">
+    <mergeCell ref="B6:B16"/>
+    <mergeCell ref="C4:C5"/>
+    <mergeCell ref="D4:D5"/>
+    <mergeCell ref="E4:G4"/>
+    <mergeCell ref="H4:H5"/>
     <mergeCell ref="J4:L4"/>
     <mergeCell ref="C1:F1"/>
     <mergeCell ref="A2:O2"/>
@@ -7336,11 +7341,6 @@
     <mergeCell ref="O4:O5"/>
     <mergeCell ref="I4:I5"/>
     <mergeCell ref="M4:M5"/>
-    <mergeCell ref="B6:B16"/>
-    <mergeCell ref="C4:C5"/>
-    <mergeCell ref="D4:D5"/>
-    <mergeCell ref="E4:G4"/>
-    <mergeCell ref="H4:H5"/>
   </mergeCells>
   <phoneticPr fontId="6" type="noConversion"/>
   <pageMargins left="0.70866141732283472" right="0.70866141732283472" top="0.74803149606299213" bottom="0.74803149606299213" header="0.31496062992125984" footer="0.31496062992125984"/>
@@ -7357,24 +7357,24 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{813C0327-CFDD-498C-87C1-8E379F217A35}">
   <dimension ref="A3:D10"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="15.5" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="14.7109375" style="130" customWidth="1"/>
-    <col min="2" max="2" width="15.28515625" style="130" customWidth="1"/>
-    <col min="3" max="3" width="13.42578125" style="130" customWidth="1"/>
-    <col min="4" max="4" width="21.28515625" style="130" customWidth="1"/>
-    <col min="5" max="16384" width="9.140625" style="130"/>
+    <col min="1" max="1" width="14.7265625" style="130" customWidth="1"/>
+    <col min="2" max="2" width="15.26953125" style="130" customWidth="1"/>
+    <col min="3" max="3" width="13.453125" style="130" customWidth="1"/>
+    <col min="4" max="4" width="21.26953125" style="130" customWidth="1"/>
+    <col min="5" max="16384" width="9.1796875" style="130"/>
   </cols>
   <sheetData>
-    <row r="3" spans="1:4" ht="32.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="283" t="s">
+    <row r="3" spans="1:4" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="293" t="s">
         <v>37</v>
       </c>
-      <c r="B3" s="283"/>
-      <c r="C3" s="283"/>
-      <c r="D3" s="283"/>
-    </row>
-    <row r="5" spans="1:4" ht="67.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B3" s="293"/>
+      <c r="C3" s="293"/>
+      <c r="D3" s="293"/>
+    </row>
+    <row r="5" spans="1:4" ht="67.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="131" t="s">
         <v>94</v>
       </c>
@@ -7388,7 +7388,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="6" spans="1:4" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:4" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="133">
         <f>(B6*C6*D6)/1000000</f>
         <v>1.944</v>
@@ -7403,7 +7403,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="C10" s="137"/>
     </row>
   </sheetData>
@@ -7416,26 +7416,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="453e7e53-5eb2-45cf-b2ab-34c867e554b8">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="aa0d983d-359a-438c-9953-3af1a8ac0831" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Dokumentas" ma:contentTypeID="0x010100BAB57CF81AE55C4698AAD22D302297F0" ma:contentTypeVersion="18" ma:contentTypeDescription="Kurkite naują dokumentą." ma:contentTypeScope="" ma:versionID="49ab401eb4052690d2a2629974c22fd6">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="453e7e53-5eb2-45cf-b2ab-34c867e554b8" xmlns:ns3="aa0d983d-359a-438c-9953-3af1a8ac0831" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="ab9969d50e0b13c63bc5bd0499c928dc" ns2:_="" ns3:_="">
     <xsd:import namespace="453e7e53-5eb2-45cf-b2ab-34c867e554b8"/>
@@ -7690,10 +7670,41 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="453e7e53-5eb2-45cf-b2ab-34c867e554b8">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="aa0d983d-359a-438c-9953-3af1a8ac0831" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{605DD0A7-BC00-4D8E-8AD3-26E2A9FDEA54}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A0A5B190-5FE3-4B47-B164-68F6A6922F48}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="453e7e53-5eb2-45cf-b2ab-34c867e554b8"/>
+    <ds:schemaRef ds:uri="aa0d983d-359a-438c-9953-3af1a8ac0831"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -7710,5 +7721,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A0A5B190-5FE3-4B47-B164-68F6A6922F48}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{605DD0A7-BC00-4D8E-8AD3-26E2A9FDEA54}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Pavadinimai1Funkcija pridėtas Pito vamzdelių koeficientų parinkimas
</commit_message>
<xml_diff>
--- a/Ivestis.xlsx
+++ b/Ivestis.xlsx
@@ -2807,6 +2807,23 @@
     <xf numFmtId="169" fontId="4" fillId="2" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
@@ -2841,23 +2858,6 @@
     </xf>
     <xf numFmtId="0" fontId="26" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
@@ -6898,49 +6898,49 @@
       <c r="O2" s="276"/>
     </row>
     <row r="4" spans="1:16" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="280" t="s">
+      <c r="A4" s="285" t="s">
         <v>80</v>
       </c>
-      <c r="B4" s="280" t="s">
+      <c r="B4" s="285" t="s">
         <v>9</v>
       </c>
-      <c r="C4" s="291" t="s">
+      <c r="C4" s="282" t="s">
         <v>81</v>
       </c>
-      <c r="D4" s="291" t="s">
+      <c r="D4" s="282" t="s">
         <v>82</v>
       </c>
-      <c r="E4" s="291" t="s">
+      <c r="E4" s="282" t="s">
         <v>83</v>
       </c>
-      <c r="F4" s="291"/>
-      <c r="G4" s="291"/>
-      <c r="H4" s="291" t="s">
+      <c r="F4" s="282"/>
+      <c r="G4" s="282"/>
+      <c r="H4" s="282" t="s">
         <v>13</v>
       </c>
-      <c r="I4" s="284" t="s">
+      <c r="I4" s="289" t="s">
         <v>84</v>
       </c>
-      <c r="J4" s="279" t="s">
+      <c r="J4" s="284" t="s">
         <v>85</v>
       </c>
-      <c r="K4" s="279"/>
-      <c r="L4" s="279"/>
-      <c r="M4" s="286" t="s">
+      <c r="K4" s="284"/>
+      <c r="L4" s="284"/>
+      <c r="M4" s="291" t="s">
         <v>86</v>
       </c>
-      <c r="N4" s="279" t="s">
+      <c r="N4" s="284" t="s">
         <v>13</v>
       </c>
-      <c r="O4" s="282" t="s">
+      <c r="O4" s="287" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="5" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="281"/>
-      <c r="B5" s="281"/>
-      <c r="C5" s="292"/>
-      <c r="D5" s="291"/>
+      <c r="A5" s="286"/>
+      <c r="B5" s="286"/>
+      <c r="C5" s="283"/>
+      <c r="D5" s="282"/>
       <c r="E5" s="146">
         <v>1</v>
       </c>
@@ -6950,8 +6950,8 @@
       <c r="G5" s="146">
         <v>3</v>
       </c>
-      <c r="H5" s="291"/>
-      <c r="I5" s="285"/>
+      <c r="H5" s="282"/>
+      <c r="I5" s="290"/>
       <c r="J5" s="12">
         <v>1</v>
       </c>
@@ -6961,16 +6961,16 @@
       <c r="L5" s="12">
         <v>3</v>
       </c>
-      <c r="M5" s="287"/>
-      <c r="N5" s="279"/>
-      <c r="O5" s="283"/>
+      <c r="M5" s="292"/>
+      <c r="N5" s="284"/>
+      <c r="O5" s="288"/>
     </row>
     <row r="6" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="170" t="str">
         <f>Paėmimas!B6</f>
         <v>3</v>
       </c>
-      <c r="B6" s="288" t="str">
+      <c r="B6" s="279" t="str">
         <f>Paėmimas!C6</f>
         <v>UAB ,,Ekopartneris", L. Ivinskio g. 65, Kaunas. Katilinė. Taršos šaltinis  Nr. 001.</v>
       </c>
@@ -7019,7 +7019,7 @@
     </row>
     <row r="7" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="32"/>
-      <c r="B7" s="289"/>
+      <c r="B7" s="280"/>
       <c r="C7" s="31"/>
       <c r="D7" s="28"/>
       <c r="E7" s="231"/>
@@ -7039,7 +7039,7 @@
     </row>
     <row r="8" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="32"/>
-      <c r="B8" s="289"/>
+      <c r="B8" s="280"/>
       <c r="C8" s="31"/>
       <c r="D8" s="106"/>
       <c r="E8" s="231"/>
@@ -7059,7 +7059,7 @@
     </row>
     <row r="9" spans="1:16" ht="17" x14ac:dyDescent="0.45">
       <c r="A9" s="32"/>
-      <c r="B9" s="289"/>
+      <c r="B9" s="280"/>
       <c r="C9" s="31">
         <v>2</v>
       </c>
@@ -7096,7 +7096,7 @@
     </row>
     <row r="10" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A10" s="32"/>
-      <c r="B10" s="289"/>
+      <c r="B10" s="280"/>
       <c r="C10" s="31"/>
       <c r="D10" s="106"/>
       <c r="E10" s="231"/>
@@ -7113,7 +7113,7 @@
     </row>
     <row r="11" spans="1:16" ht="17" x14ac:dyDescent="0.45">
       <c r="A11" s="32"/>
-      <c r="B11" s="289"/>
+      <c r="B11" s="280"/>
       <c r="C11" s="31">
         <v>41</v>
       </c>
@@ -7149,7 +7149,7 @@
     </row>
     <row r="12" spans="1:16" ht="30.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A12" s="32"/>
-      <c r="B12" s="289"/>
+      <c r="B12" s="280"/>
       <c r="C12" s="138" t="s">
         <v>41</v>
       </c>
@@ -7185,7 +7185,7 @@
     </row>
     <row r="13" spans="1:16" ht="17" x14ac:dyDescent="0.45">
       <c r="A13" s="32"/>
-      <c r="B13" s="289"/>
+      <c r="B13" s="280"/>
       <c r="C13" s="139" t="s">
         <v>42</v>
       </c>
@@ -7221,7 +7221,7 @@
     </row>
     <row r="14" spans="1:16" ht="17" x14ac:dyDescent="0.45">
       <c r="A14" s="32"/>
-      <c r="B14" s="289"/>
+      <c r="B14" s="280"/>
       <c r="C14" s="139" t="s">
         <v>43</v>
       </c>
@@ -7257,7 +7257,7 @@
     </row>
     <row r="15" spans="1:16" ht="17" x14ac:dyDescent="0.45">
       <c r="A15" s="32"/>
-      <c r="B15" s="289"/>
+      <c r="B15" s="280"/>
       <c r="C15" s="140" t="s">
         <v>44</v>
       </c>
@@ -7293,7 +7293,7 @@
     </row>
     <row r="16" spans="1:16" ht="32.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A16" s="22"/>
-      <c r="B16" s="290"/>
+      <c r="B16" s="281"/>
       <c r="C16" s="31"/>
       <c r="D16" s="109"/>
       <c r="E16" s="21"/>
@@ -7327,11 +7327,6 @@
     </sortState>
   </autoFilter>
   <mergeCells count="14">
-    <mergeCell ref="B6:B16"/>
-    <mergeCell ref="C4:C5"/>
-    <mergeCell ref="D4:D5"/>
-    <mergeCell ref="E4:G4"/>
-    <mergeCell ref="H4:H5"/>
     <mergeCell ref="J4:L4"/>
     <mergeCell ref="C1:F1"/>
     <mergeCell ref="A2:O2"/>
@@ -7341,6 +7336,11 @@
     <mergeCell ref="O4:O5"/>
     <mergeCell ref="I4:I5"/>
     <mergeCell ref="M4:M5"/>
+    <mergeCell ref="B6:B16"/>
+    <mergeCell ref="C4:C5"/>
+    <mergeCell ref="D4:D5"/>
+    <mergeCell ref="E4:G4"/>
+    <mergeCell ref="H4:H5"/>
   </mergeCells>
   <phoneticPr fontId="6" type="noConversion"/>
   <pageMargins left="0.70866141732283472" right="0.70866141732283472" top="0.74803149606299213" bottom="0.74803149606299213" header="0.31496062992125984" footer="0.31496062992125984"/>
@@ -7671,6 +7671,15 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <lcf76f155ced4ddcb4097134ff3c332f xmlns="453e7e53-5eb2-45cf-b2ab-34c867e554b8">
@@ -7679,15 +7688,6 @@
     <TaxCatchAll xmlns="aa0d983d-359a-438c-9953-3af1a8ac0831" xsi:nil="true"/>
   </documentManagement>
 </p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -7710,6 +7710,14 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{605DD0A7-BC00-4D8E-8AD3-26E2A9FDEA54}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{709F4DDD-DF1A-450D-8BF1-976CA47CFD58}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
@@ -7718,12 +7726,4 @@
     <ds:schemaRef ds:uri="aa0d983d-359a-438c-9953-3af1a8ac0831"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{605DD0A7-BC00-4D8E-8AD3-26E2A9FDEA54}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Pridįtas Skesrpjūvio ploto skaičiavimas
</commit_message>
<xml_diff>
--- a/Ivestis.xlsx
+++ b/Ivestis.xlsx
@@ -10,7 +10,7 @@
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="263" documentId="13_ncr:1_{D8ED3FA4-1188-4E70-924F-660A50F19C4F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8685D0F3-FD86-4775-8711-4CB6F11BBCB9}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" tabRatio="821" firstSheet="1" activeTab="7" xr2:uid="{B097D0E3-85A4-46F7-964F-ABE00A6941B9}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" tabRatio="821" firstSheet="1" activeTab="3" xr2:uid="{B097D0E3-85A4-46F7-964F-ABE00A6941B9}"/>
   </bookViews>
   <sheets>
     <sheet name="Compatibility Report" sheetId="4" state="hidden" r:id="rId1"/>
@@ -2668,6 +2668,86 @@
     <xf numFmtId="164" fontId="4" fillId="2" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="10" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="10" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="14" fontId="30" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="2" fontId="9" fillId="8" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="2" fontId="9" fillId="8" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="2" fontId="9" fillId="8" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
@@ -2696,82 +2776,6 @@
       <alignment horizontal="center" vertical="top" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="49" fontId="10" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="49" fontId="10" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="14" fontId="30" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="2" fontId="9" fillId="8" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="2" fontId="9" fillId="8" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="2" fontId="9" fillId="8" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" wrapText="1"/>
       <protection locked="0"/>
@@ -2807,6 +2811,42 @@
     <xf numFmtId="169" fontId="4" fillId="2" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="7" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
@@ -2822,46 +2862,6 @@
     </xf>
     <xf numFmtId="0" fontId="8" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="7" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
   </cellXfs>
@@ -3293,31 +3293,31 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="D2" s="252" t="s">
+      <c r="D2" s="246" t="s">
         <v>108</v>
       </c>
-      <c r="E2" s="252"/>
-      <c r="F2" s="252"/>
-      <c r="G2" s="252"/>
-      <c r="H2" s="252"/>
-      <c r="I2" s="252"/>
-      <c r="J2" s="252"/>
-      <c r="K2" s="252"/>
-      <c r="L2" s="252"/>
-      <c r="M2" s="252"/>
-      <c r="N2" s="252"/>
-      <c r="O2" s="252"/>
-      <c r="P2" s="252"/>
-      <c r="Q2" s="252"/>
-      <c r="R2" s="252"/>
-      <c r="S2" s="252"/>
-      <c r="T2" s="252"/>
-      <c r="U2" s="252"/>
-      <c r="V2" s="252"/>
-      <c r="W2" s="252"/>
-      <c r="X2" s="252"/>
-      <c r="Y2" s="252"/>
-      <c r="Z2" s="252"/>
+      <c r="E2" s="246"/>
+      <c r="F2" s="246"/>
+      <c r="G2" s="246"/>
+      <c r="H2" s="246"/>
+      <c r="I2" s="246"/>
+      <c r="J2" s="246"/>
+      <c r="K2" s="246"/>
+      <c r="L2" s="246"/>
+      <c r="M2" s="246"/>
+      <c r="N2" s="246"/>
+      <c r="O2" s="246"/>
+      <c r="P2" s="246"/>
+      <c r="Q2" s="246"/>
+      <c r="R2" s="246"/>
+      <c r="S2" s="246"/>
+      <c r="T2" s="246"/>
+      <c r="U2" s="246"/>
+      <c r="V2" s="246"/>
+      <c r="W2" s="246"/>
+      <c r="X2" s="246"/>
+      <c r="Y2" s="246"/>
+      <c r="Z2" s="246"/>
     </row>
     <row r="4" spans="1:28" s="10" customFormat="1" ht="126" x14ac:dyDescent="0.25">
       <c r="A4" s="9" t="s">
@@ -3406,13 +3406,13 @@
       </c>
     </row>
     <row r="5" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A5" s="253">
+      <c r="A5" s="247">
         <v>46063</v>
       </c>
-      <c r="B5" s="256">
+      <c r="B5" s="250">
         <v>5</v>
       </c>
-      <c r="C5" s="259" t="s">
+      <c r="C5" s="253" t="s">
         <v>140</v>
       </c>
       <c r="D5" s="177">
@@ -3503,14 +3503,14 @@
         <f>Aerodinamika!G27</f>
         <v>1.3179692000000001</v>
       </c>
-      <c r="AB5" s="250" t="s">
+      <c r="AB5" s="244" t="s">
         <v>139</v>
       </c>
     </row>
     <row r="6" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A6" s="254"/>
-      <c r="B6" s="257"/>
-      <c r="C6" s="260"/>
+      <c r="A6" s="248"/>
+      <c r="B6" s="251"/>
+      <c r="C6" s="254"/>
       <c r="D6" s="177">
         <v>16</v>
       </c>
@@ -3595,12 +3595,12 @@
         <f>O5*X6</f>
         <v>0.79775867584824989</v>
       </c>
-      <c r="AB6" s="251"/>
+      <c r="AB6" s="245"/>
     </row>
     <row r="7" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A7" s="254"/>
-      <c r="B7" s="257"/>
-      <c r="C7" s="260"/>
+      <c r="A7" s="248"/>
+      <c r="B7" s="251"/>
+      <c r="C7" s="254"/>
       <c r="D7" s="200">
         <v>31</v>
       </c>
@@ -3651,9 +3651,9 @@
       <c r="S7" s="176"/>
     </row>
     <row r="8" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A8" s="254"/>
-      <c r="B8" s="257"/>
-      <c r="C8" s="260"/>
+      <c r="A8" s="248"/>
+      <c r="B8" s="251"/>
+      <c r="C8" s="254"/>
       <c r="D8" s="177">
         <v>60</v>
       </c>
@@ -3708,9 +3708,9 @@
       </c>
     </row>
     <row r="9" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A9" s="254"/>
-      <c r="B9" s="257"/>
-      <c r="C9" s="260"/>
+      <c r="A9" s="248"/>
+      <c r="B9" s="251"/>
+      <c r="C9" s="254"/>
       <c r="D9" s="177">
         <v>89</v>
       </c>
@@ -3754,9 +3754,9 @@
       </c>
     </row>
     <row r="10" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A10" s="254"/>
-      <c r="B10" s="257"/>
-      <c r="C10" s="260"/>
+      <c r="A10" s="248"/>
+      <c r="B10" s="251"/>
+      <c r="C10" s="254"/>
       <c r="D10" s="177">
         <v>104</v>
       </c>
@@ -3800,9 +3800,9 @@
       </c>
     </row>
     <row r="11" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A11" s="255"/>
-      <c r="B11" s="258"/>
-      <c r="C11" s="261"/>
+      <c r="A11" s="249"/>
+      <c r="B11" s="252"/>
+      <c r="C11" s="255"/>
       <c r="D11" s="177">
         <v>115</v>
       </c>
@@ -3871,18 +3871,18 @@
       <c r="D13" s="200" t="s">
         <v>135</v>
       </c>
-      <c r="E13" s="262" t="s">
+      <c r="E13" s="256" t="s">
         <v>136</v>
       </c>
-      <c r="F13" s="263"/>
-      <c r="G13" s="263"/>
-      <c r="H13" s="263"/>
-      <c r="I13" s="263"/>
-      <c r="J13" s="263"/>
-      <c r="K13" s="263"/>
-      <c r="L13" s="263"/>
-      <c r="M13" s="263"/>
-      <c r="N13" s="264"/>
+      <c r="F13" s="257"/>
+      <c r="G13" s="257"/>
+      <c r="H13" s="257"/>
+      <c r="I13" s="257"/>
+      <c r="J13" s="257"/>
+      <c r="K13" s="257"/>
+      <c r="L13" s="257"/>
+      <c r="M13" s="257"/>
+      <c r="N13" s="258"/>
     </row>
     <row r="14" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A14" s="206"/>
@@ -3917,31 +3917,31 @@
       <c r="A17" s="206"/>
       <c r="B17" s="206"/>
       <c r="C17" s="206"/>
-      <c r="D17" s="265" t="s">
+      <c r="D17" s="259" t="s">
         <v>138</v>
       </c>
-      <c r="E17" s="252"/>
-      <c r="F17" s="252"/>
-      <c r="G17" s="252"/>
-      <c r="H17" s="252"/>
-      <c r="I17" s="252"/>
-      <c r="J17" s="252"/>
-      <c r="K17" s="252"/>
-      <c r="L17" s="252"/>
-      <c r="M17" s="252"/>
-      <c r="N17" s="252"/>
-      <c r="O17" s="252"/>
-      <c r="P17" s="252"/>
-      <c r="Q17" s="252"/>
-      <c r="R17" s="252"/>
-      <c r="S17" s="252"/>
-      <c r="T17" s="252"/>
-      <c r="U17" s="252"/>
-      <c r="V17" s="252"/>
-      <c r="W17" s="252"/>
-      <c r="X17" s="252"/>
-      <c r="Y17" s="252"/>
-      <c r="Z17" s="252"/>
+      <c r="E17" s="246"/>
+      <c r="F17" s="246"/>
+      <c r="G17" s="246"/>
+      <c r="H17" s="246"/>
+      <c r="I17" s="246"/>
+      <c r="J17" s="246"/>
+      <c r="K17" s="246"/>
+      <c r="L17" s="246"/>
+      <c r="M17" s="246"/>
+      <c r="N17" s="246"/>
+      <c r="O17" s="246"/>
+      <c r="P17" s="246"/>
+      <c r="Q17" s="246"/>
+      <c r="R17" s="246"/>
+      <c r="S17" s="246"/>
+      <c r="T17" s="246"/>
+      <c r="U17" s="246"/>
+      <c r="V17" s="246"/>
+      <c r="W17" s="246"/>
+      <c r="X17" s="246"/>
+      <c r="Y17" s="246"/>
+      <c r="Z17" s="246"/>
     </row>
     <row r="18" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A18" s="206"/>
@@ -4047,9 +4047,9 @@
       </c>
     </row>
     <row r="20" spans="1:28" ht="16" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="266"/>
-      <c r="B20" s="266"/>
-      <c r="C20" s="266"/>
+      <c r="A20" s="260"/>
+      <c r="B20" s="260"/>
+      <c r="C20" s="260"/>
       <c r="D20" s="177">
         <v>3</v>
       </c>
@@ -4126,12 +4126,12 @@
       <c r="AA20" s="219">
         <v>1.35</v>
       </c>
-      <c r="AB20" s="250"/>
+      <c r="AB20" s="244"/>
     </row>
     <row r="21" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A21" s="267"/>
-      <c r="B21" s="267"/>
-      <c r="C21" s="267"/>
+      <c r="A21" s="261"/>
+      <c r="B21" s="261"/>
+      <c r="C21" s="261"/>
       <c r="D21" s="177">
         <v>15</v>
       </c>
@@ -4202,12 +4202,12 @@
         <f>O20*X21</f>
         <v>1.0671545706141219</v>
       </c>
-      <c r="AB21" s="251"/>
+      <c r="AB21" s="245"/>
     </row>
     <row r="22" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A22" s="267"/>
-      <c r="B22" s="267"/>
-      <c r="C22" s="267"/>
+      <c r="A22" s="261"/>
+      <c r="B22" s="261"/>
+      <c r="C22" s="261"/>
       <c r="D22" s="200">
         <v>27</v>
       </c>
@@ -4246,9 +4246,9 @@
       <c r="S22" s="176"/>
     </row>
     <row r="23" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A23" s="267"/>
-      <c r="B23" s="267"/>
-      <c r="C23" s="267"/>
+      <c r="A23" s="261"/>
+      <c r="B23" s="261"/>
+      <c r="C23" s="261"/>
       <c r="D23" s="177">
         <v>4</v>
       </c>
@@ -4291,9 +4291,9 @@
       </c>
     </row>
     <row r="24" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A24" s="267"/>
-      <c r="B24" s="267"/>
-      <c r="C24" s="267"/>
+      <c r="A24" s="261"/>
+      <c r="B24" s="261"/>
+      <c r="C24" s="261"/>
       <c r="D24" s="177">
         <v>5</v>
       </c>
@@ -4325,9 +4325,9 @@
       </c>
     </row>
     <row r="25" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A25" s="267"/>
-      <c r="B25" s="267"/>
-      <c r="C25" s="267"/>
+      <c r="A25" s="261"/>
+      <c r="B25" s="261"/>
+      <c r="C25" s="261"/>
       <c r="D25" s="177">
         <v>6</v>
       </c>
@@ -4359,9 +4359,9 @@
       </c>
     </row>
     <row r="26" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A26" s="268"/>
-      <c r="B26" s="268"/>
-      <c r="C26" s="268"/>
+      <c r="A26" s="262"/>
+      <c r="B26" s="262"/>
+      <c r="C26" s="262"/>
       <c r="D26" s="177">
         <v>7</v>
       </c>
@@ -4451,18 +4451,18 @@
       <c r="I2" s="10"/>
     </row>
     <row r="3" spans="1:12" ht="23.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="243" t="s">
+      <c r="A3" s="263" t="s">
         <v>107</v>
       </c>
-      <c r="B3" s="243"/>
-      <c r="C3" s="243"/>
-      <c r="D3" s="243"/>
-      <c r="E3" s="243"/>
-      <c r="F3" s="243"/>
-      <c r="G3" s="243"/>
-      <c r="H3" s="243"/>
-      <c r="I3" s="243"/>
-      <c r="J3" s="243"/>
+      <c r="B3" s="263"/>
+      <c r="C3" s="263"/>
+      <c r="D3" s="263"/>
+      <c r="E3" s="263"/>
+      <c r="F3" s="263"/>
+      <c r="G3" s="263"/>
+      <c r="H3" s="263"/>
+      <c r="I3" s="263"/>
+      <c r="J3" s="263"/>
     </row>
     <row r="4" spans="1:12" ht="14" x14ac:dyDescent="0.3">
       <c r="A4" s="10"/>
@@ -4609,46 +4609,46 @@
       <c r="L10" s="45"/>
     </row>
     <row r="11" spans="1:12" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="H11" s="244" t="s">
+      <c r="H11" s="264" t="s">
         <v>26</v>
       </c>
-      <c r="I11" s="247" t="s">
+      <c r="I11" s="267" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="12" spans="1:12" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="H12" s="245"/>
-      <c r="I12" s="248"/>
+      <c r="H12" s="265"/>
+      <c r="I12" s="268"/>
     </row>
     <row r="13" spans="1:12" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="H13" s="245"/>
-      <c r="I13" s="248"/>
+      <c r="H13" s="265"/>
+      <c r="I13" s="268"/>
     </row>
     <row r="14" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="H14" s="245"/>
-      <c r="I14" s="248"/>
+      <c r="H14" s="265"/>
+      <c r="I14" s="268"/>
     </row>
     <row r="15" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="H15" s="245"/>
-      <c r="I15" s="248"/>
+      <c r="H15" s="265"/>
+      <c r="I15" s="268"/>
     </row>
     <row r="16" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="H16" s="245"/>
-      <c r="I16" s="248"/>
+      <c r="H16" s="265"/>
+      <c r="I16" s="268"/>
     </row>
     <row r="17" spans="8:9" x14ac:dyDescent="0.3">
-      <c r="H17" s="245"/>
-      <c r="I17" s="248"/>
+      <c r="H17" s="265"/>
+      <c r="I17" s="268"/>
     </row>
     <row r="18" spans="8:9" x14ac:dyDescent="0.3">
-      <c r="H18" s="246"/>
-      <c r="I18" s="248"/>
+      <c r="H18" s="266"/>
+      <c r="I18" s="268"/>
     </row>
     <row r="19" spans="8:9" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="I19" s="248"/>
+      <c r="I19" s="268"/>
     </row>
     <row r="20" spans="8:9" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="I20" s="249"/>
+      <c r="I20" s="269"/>
     </row>
     <row r="21" spans="8:9" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="I21" s="57"/>
@@ -4710,35 +4710,35 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:22" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C1" s="274" t="s">
+      <c r="C1" s="275" t="s">
         <v>14</v>
       </c>
-      <c r="D1" s="274"/>
+      <c r="D1" s="275"/>
       <c r="E1" s="15"/>
       <c r="S1" s="16"/>
     </row>
     <row r="2" spans="1:22" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="275" t="s">
+      <c r="A2" s="276" t="s">
         <v>97</v>
       </c>
-      <c r="B2" s="275"/>
-      <c r="C2" s="275"/>
-      <c r="D2" s="275"/>
-      <c r="E2" s="275"/>
-      <c r="F2" s="275"/>
-      <c r="G2" s="275"/>
-      <c r="H2" s="275"/>
-      <c r="I2" s="275"/>
-      <c r="J2" s="275"/>
-      <c r="K2" s="275"/>
-      <c r="L2" s="275"/>
-      <c r="M2" s="275"/>
-      <c r="N2" s="275"/>
-      <c r="O2" s="275"/>
-      <c r="P2" s="275"/>
-      <c r="Q2" s="275"/>
-      <c r="R2" s="275"/>
-      <c r="S2" s="275"/>
+      <c r="B2" s="276"/>
+      <c r="C2" s="276"/>
+      <c r="D2" s="276"/>
+      <c r="E2" s="276"/>
+      <c r="F2" s="276"/>
+      <c r="G2" s="276"/>
+      <c r="H2" s="276"/>
+      <c r="I2" s="276"/>
+      <c r="J2" s="276"/>
+      <c r="K2" s="276"/>
+      <c r="L2" s="276"/>
+      <c r="M2" s="276"/>
+      <c r="N2" s="276"/>
+      <c r="O2" s="276"/>
+      <c r="P2" s="276"/>
+      <c r="Q2" s="276"/>
+      <c r="R2" s="276"/>
+      <c r="S2" s="276"/>
     </row>
     <row r="3" spans="1:22" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="17"/>
@@ -4840,7 +4840,7 @@
       <c r="B6" s="229" t="s">
         <v>141</v>
       </c>
-      <c r="C6" s="270" t="str">
+      <c r="C6" s="271" t="str">
         <f>Greitis!C5</f>
         <v>UAB ,,Ekopartneris", L. Ivinskio g. 65, Kaunas. Katilinė. Taršos šaltinis  Nr. 001.</v>
       </c>
@@ -4912,7 +4912,7 @@
     <row r="7" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A7" s="225"/>
       <c r="B7" s="226"/>
-      <c r="C7" s="271"/>
+      <c r="C7" s="272"/>
       <c r="D7" s="19"/>
       <c r="E7" s="20"/>
       <c r="F7" s="78">
@@ -4975,7 +4975,7 @@
     <row r="8" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A8" s="225"/>
       <c r="B8" s="226"/>
-      <c r="C8" s="271"/>
+      <c r="C8" s="272"/>
       <c r="D8" s="19"/>
       <c r="E8" s="20"/>
       <c r="F8" s="78">
@@ -5038,7 +5038,7 @@
     <row r="9" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A9" s="227"/>
       <c r="B9" s="227"/>
-      <c r="C9" s="271"/>
+      <c r="C9" s="272"/>
       <c r="D9" s="49"/>
       <c r="E9" s="49"/>
       <c r="F9" s="78">
@@ -5104,7 +5104,7 @@
     <row r="10" spans="1:22" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="227"/>
       <c r="B10" s="227"/>
-      <c r="C10" s="271"/>
+      <c r="C10" s="272"/>
       <c r="D10" s="49"/>
       <c r="E10" s="49"/>
       <c r="F10" s="78">
@@ -5154,20 +5154,20 @@
       </c>
       <c r="R10" s="49"/>
       <c r="S10" s="49"/>
-      <c r="T10" s="273" t="s">
+      <c r="T10" s="274" t="s">
         <v>28</v>
       </c>
-      <c r="U10" s="273" t="s">
+      <c r="U10" s="274" t="s">
         <v>29</v>
       </c>
-      <c r="V10" s="269" t="s">
+      <c r="V10" s="270" t="s">
         <v>36</v>
       </c>
     </row>
     <row r="11" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A11" s="227"/>
       <c r="B11" s="227"/>
-      <c r="C11" s="271"/>
+      <c r="C11" s="272"/>
       <c r="D11" s="49"/>
       <c r="E11" s="49"/>
       <c r="F11" s="78">
@@ -5217,14 +5217,14 @@
       </c>
       <c r="R11" s="49"/>
       <c r="S11" s="49"/>
-      <c r="T11" s="273"/>
-      <c r="U11" s="273"/>
-      <c r="V11" s="269"/>
+      <c r="T11" s="274"/>
+      <c r="U11" s="274"/>
+      <c r="V11" s="270"/>
     </row>
     <row r="12" spans="1:22" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="228"/>
       <c r="B12" s="228"/>
-      <c r="C12" s="272"/>
+      <c r="C12" s="273"/>
       <c r="D12" s="34"/>
       <c r="E12" s="34"/>
       <c r="F12" s="78">
@@ -5274,9 +5274,9 @@
       </c>
       <c r="R12" s="34"/>
       <c r="S12" s="34"/>
-      <c r="T12" s="273"/>
-      <c r="U12" s="273"/>
-      <c r="V12" s="269"/>
+      <c r="T12" s="274"/>
+      <c r="U12" s="274"/>
+      <c r="V12" s="270"/>
     </row>
     <row r="13" spans="1:22" x14ac:dyDescent="0.3">
       <c r="L13" s="81">
@@ -5317,7 +5317,7 @@
         <f t="shared" si="21"/>
         <v>3</v>
       </c>
-      <c r="C17" s="270" t="str">
+      <c r="C17" s="271" t="str">
         <f t="shared" si="21"/>
         <v>UAB ,,Ekopartneris", L. Ivinskio g. 65, Kaunas. Katilinė. Taršos šaltinis  Nr. 001.</v>
       </c>
@@ -5385,7 +5385,7 @@
     <row r="18" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A18" s="35"/>
       <c r="B18" s="32"/>
-      <c r="C18" s="271"/>
+      <c r="C18" s="272"/>
       <c r="D18" s="19"/>
       <c r="E18" s="20"/>
       <c r="F18" s="78">
@@ -5439,7 +5439,7 @@
     <row r="19" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A19" s="35"/>
       <c r="B19" s="32"/>
-      <c r="C19" s="271"/>
+      <c r="C19" s="272"/>
       <c r="D19" s="19"/>
       <c r="E19" s="20"/>
       <c r="F19" s="78">
@@ -5493,7 +5493,7 @@
     <row r="20" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A20" s="49"/>
       <c r="B20" s="49"/>
-      <c r="C20" s="271"/>
+      <c r="C20" s="272"/>
       <c r="D20" s="49"/>
       <c r="E20" s="49"/>
       <c r="F20" s="78">
@@ -5547,7 +5547,7 @@
     <row r="21" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A21" s="49"/>
       <c r="B21" s="49"/>
-      <c r="C21" s="271"/>
+      <c r="C21" s="272"/>
       <c r="D21" s="49"/>
       <c r="E21" s="49"/>
       <c r="F21" s="78">
@@ -5601,7 +5601,7 @@
     <row r="22" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A22" s="49"/>
       <c r="B22" s="49"/>
-      <c r="C22" s="271"/>
+      <c r="C22" s="272"/>
       <c r="D22" s="49"/>
       <c r="E22" s="49"/>
       <c r="F22" s="78">
@@ -5655,7 +5655,7 @@
     <row r="23" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A23" s="34"/>
       <c r="B23" s="34"/>
-      <c r="C23" s="272"/>
+      <c r="C23" s="273"/>
       <c r="D23" s="34"/>
       <c r="E23" s="34"/>
       <c r="F23" s="78">
@@ -5824,26 +5824,26 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:17" ht="30.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C1" s="274" t="s">
+      <c r="C1" s="275" t="s">
         <v>15</v>
       </c>
-      <c r="D1" s="274"/>
+      <c r="D1" s="275"/>
       <c r="Q1" s="16"/>
     </row>
     <row r="2" spans="1:17" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C2" s="276" t="s">
+      <c r="C2" s="277" t="s">
         <v>98</v>
       </c>
-      <c r="D2" s="276"/>
-      <c r="E2" s="276"/>
-      <c r="F2" s="276"/>
-      <c r="G2" s="276"/>
-      <c r="H2" s="276"/>
-      <c r="I2" s="276"/>
-      <c r="J2" s="276"/>
-      <c r="K2" s="276"/>
-      <c r="L2" s="276"/>
-      <c r="M2" s="276"/>
+      <c r="D2" s="277"/>
+      <c r="E2" s="277"/>
+      <c r="F2" s="277"/>
+      <c r="G2" s="277"/>
+      <c r="H2" s="277"/>
+      <c r="I2" s="277"/>
+      <c r="J2" s="277"/>
+      <c r="K2" s="277"/>
+      <c r="L2" s="277"/>
+      <c r="M2" s="277"/>
       <c r="Q2" s="16"/>
     </row>
     <row r="3" spans="1:17" ht="12" customHeight="1" x14ac:dyDescent="0.3">
@@ -5905,7 +5905,7 @@
         <f>Paėmimas!B6</f>
         <v>3</v>
       </c>
-      <c r="C6" s="270" t="str">
+      <c r="C6" s="271" t="str">
         <f>Paėmimas!C6</f>
         <v>UAB ,,Ekopartneris", L. Ivinskio g. 65, Kaunas. Katilinė. Taršos šaltinis  Nr. 001.</v>
       </c>
@@ -5957,7 +5957,7 @@
     <row r="7" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="59"/>
       <c r="B7" s="23"/>
-      <c r="C7" s="271"/>
+      <c r="C7" s="272"/>
       <c r="D7" s="58">
         <f>Paėmimas!L7</f>
         <v>3.5999999999999997E-2</v>
@@ -5994,7 +5994,7 @@
     <row r="8" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="59"/>
       <c r="B8" s="23"/>
-      <c r="C8" s="271"/>
+      <c r="C8" s="272"/>
       <c r="D8" s="58">
         <f>Paėmimas!L8</f>
         <v>3.5999999999999997E-2</v>
@@ -6031,7 +6031,7 @@
     <row r="9" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="59"/>
       <c r="B9" s="23"/>
-      <c r="C9" s="271"/>
+      <c r="C9" s="272"/>
       <c r="D9" s="58">
         <f>Paėmimas!L9</f>
         <v>3.5999999999999997E-2</v>
@@ -6068,7 +6068,7 @@
     <row r="10" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="59"/>
       <c r="B10" s="23"/>
-      <c r="C10" s="271"/>
+      <c r="C10" s="272"/>
       <c r="D10" s="58">
         <f>Paėmimas!L10</f>
         <v>3.5999999999999997E-2</v>
@@ -6105,7 +6105,7 @@
     <row r="11" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="59"/>
       <c r="B11" s="23"/>
-      <c r="C11" s="271"/>
+      <c r="C11" s="272"/>
       <c r="D11" s="58">
         <f>Paėmimas!L11</f>
         <v>3.3000000000000002E-2</v>
@@ -6142,7 +6142,7 @@
     <row r="12" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="61"/>
       <c r="B12" s="62"/>
-      <c r="C12" s="271"/>
+      <c r="C12" s="272"/>
       <c r="D12" s="58">
         <f>Paėmimas!L12</f>
         <v>0.03</v>
@@ -6225,7 +6225,7 @@
         <f>Paėmimas!B17</f>
         <v>3</v>
       </c>
-      <c r="C17" s="270" t="str">
+      <c r="C17" s="271" t="str">
         <f>Paėmimas!C17</f>
         <v>UAB ,,Ekopartneris", L. Ivinskio g. 65, Kaunas. Katilinė. Taršos šaltinis  Nr. 001.</v>
       </c>
@@ -6277,7 +6277,7 @@
     <row r="18" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A18" s="59"/>
       <c r="B18" s="23"/>
-      <c r="C18" s="271"/>
+      <c r="C18" s="272"/>
       <c r="D18" s="58">
         <f>Paėmimas!L18</f>
         <v>3.3000000000000002E-2</v>
@@ -6314,7 +6314,7 @@
     <row r="19" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A19" s="59"/>
       <c r="B19" s="23"/>
-      <c r="C19" s="271"/>
+      <c r="C19" s="272"/>
       <c r="D19" s="58">
         <f>Paėmimas!L19</f>
         <v>3.3000000000000002E-2</v>
@@ -6351,7 +6351,7 @@
     <row r="20" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A20" s="59"/>
       <c r="B20" s="23"/>
-      <c r="C20" s="271"/>
+      <c r="C20" s="272"/>
       <c r="D20" s="58">
         <f>Paėmimas!L20</f>
         <v>3.5999999999999997E-2</v>
@@ -6388,7 +6388,7 @@
     <row r="21" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A21" s="59"/>
       <c r="B21" s="23"/>
-      <c r="C21" s="271"/>
+      <c r="C21" s="272"/>
       <c r="D21" s="58">
         <f>Paėmimas!L21</f>
         <v>3.3000000000000002E-2</v>
@@ -6425,7 +6425,7 @@
     <row r="22" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A22" s="59"/>
       <c r="B22" s="23"/>
-      <c r="C22" s="271"/>
+      <c r="C22" s="272"/>
       <c r="D22" s="58">
         <f>Paėmimas!L22</f>
         <v>3.3000000000000002E-2</v>
@@ -6462,7 +6462,7 @@
     <row r="23" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A23" s="61"/>
       <c r="B23" s="62"/>
-      <c r="C23" s="271"/>
+      <c r="C23" s="272"/>
       <c r="D23" s="58">
         <f>Paėmimas!L23</f>
         <v>3.3000000000000002E-2</v>
@@ -6645,29 +6645,29 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:18" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C1" s="274" t="s">
+      <c r="C1" s="275" t="s">
         <v>16</v>
       </c>
-      <c r="D1" s="274"/>
+      <c r="D1" s="275"/>
       <c r="R1" s="16"/>
     </row>
     <row r="2" spans="1:18" x14ac:dyDescent="0.3">
-      <c r="A2" s="276" t="s">
+      <c r="A2" s="277" t="s">
         <v>99</v>
       </c>
-      <c r="B2" s="276"/>
-      <c r="C2" s="276"/>
-      <c r="D2" s="276"/>
-      <c r="E2" s="276"/>
-      <c r="F2" s="276"/>
-      <c r="G2" s="276"/>
-      <c r="H2" s="276"/>
-      <c r="I2" s="276"/>
-      <c r="J2" s="276"/>
-      <c r="K2" s="276"/>
-      <c r="L2" s="276"/>
-      <c r="M2" s="276"/>
-      <c r="N2" s="276"/>
+      <c r="B2" s="277"/>
+      <c r="C2" s="277"/>
+      <c r="D2" s="277"/>
+      <c r="E2" s="277"/>
+      <c r="F2" s="277"/>
+      <c r="G2" s="277"/>
+      <c r="H2" s="277"/>
+      <c r="I2" s="277"/>
+      <c r="J2" s="277"/>
+      <c r="K2" s="277"/>
+      <c r="L2" s="277"/>
+      <c r="M2" s="277"/>
+      <c r="N2" s="277"/>
       <c r="O2" s="156"/>
     </row>
     <row r="3" spans="1:18" x14ac:dyDescent="0.3">
@@ -6738,7 +6738,7 @@
         <f>Svėrimas!A6</f>
         <v>3</v>
       </c>
-      <c r="C6" s="277" t="str">
+      <c r="C6" s="278" t="str">
         <f>Paėmimas!C6</f>
         <v>UAB ,,Ekopartneris", L. Ivinskio g. 65, Kaunas. Katilinė. Taršos šaltinis  Nr. 001.</v>
       </c>
@@ -6797,7 +6797,7 @@
     <row r="7" spans="1:18" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="66"/>
       <c r="B7" s="67"/>
-      <c r="C7" s="277"/>
+      <c r="C7" s="278"/>
       <c r="D7" s="68"/>
       <c r="E7" s="127"/>
       <c r="F7" s="129"/>
@@ -6815,7 +6815,7 @@
     <row r="8" spans="1:18" ht="22.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="76"/>
       <c r="B8" s="65"/>
-      <c r="C8" s="278"/>
+      <c r="C8" s="279"/>
       <c r="D8" s="68"/>
       <c r="E8" s="127"/>
       <c r="F8" s="129"/>
@@ -6871,76 +6871,76 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:16" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C1" s="274" t="s">
+      <c r="C1" s="275" t="s">
         <v>17</v>
       </c>
-      <c r="D1" s="274"/>
-      <c r="E1" s="274"/>
-      <c r="F1" s="274"/>
+      <c r="D1" s="275"/>
+      <c r="E1" s="275"/>
+      <c r="F1" s="275"/>
     </row>
     <row r="2" spans="1:16" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="276" t="s">
+      <c r="A2" s="277" t="s">
         <v>100</v>
       </c>
-      <c r="B2" s="276"/>
-      <c r="C2" s="276"/>
-      <c r="D2" s="276"/>
-      <c r="E2" s="276"/>
-      <c r="F2" s="276"/>
-      <c r="G2" s="276"/>
-      <c r="H2" s="276"/>
-      <c r="I2" s="276"/>
-      <c r="J2" s="276"/>
-      <c r="K2" s="276"/>
-      <c r="L2" s="276"/>
-      <c r="M2" s="276"/>
-      <c r="N2" s="276"/>
-      <c r="O2" s="276"/>
+      <c r="B2" s="277"/>
+      <c r="C2" s="277"/>
+      <c r="D2" s="277"/>
+      <c r="E2" s="277"/>
+      <c r="F2" s="277"/>
+      <c r="G2" s="277"/>
+      <c r="H2" s="277"/>
+      <c r="I2" s="277"/>
+      <c r="J2" s="277"/>
+      <c r="K2" s="277"/>
+      <c r="L2" s="277"/>
+      <c r="M2" s="277"/>
+      <c r="N2" s="277"/>
+      <c r="O2" s="277"/>
     </row>
     <row r="4" spans="1:16" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="285" t="s">
+      <c r="A4" s="281" t="s">
         <v>80</v>
       </c>
-      <c r="B4" s="285" t="s">
+      <c r="B4" s="281" t="s">
         <v>9</v>
       </c>
-      <c r="C4" s="282" t="s">
+      <c r="C4" s="292" t="s">
         <v>81</v>
       </c>
-      <c r="D4" s="282" t="s">
+      <c r="D4" s="292" t="s">
         <v>82</v>
       </c>
-      <c r="E4" s="282" t="s">
+      <c r="E4" s="292" t="s">
         <v>83</v>
       </c>
-      <c r="F4" s="282"/>
-      <c r="G4" s="282"/>
-      <c r="H4" s="282" t="s">
+      <c r="F4" s="292"/>
+      <c r="G4" s="292"/>
+      <c r="H4" s="292" t="s">
         <v>13</v>
       </c>
-      <c r="I4" s="289" t="s">
+      <c r="I4" s="285" t="s">
         <v>84</v>
       </c>
-      <c r="J4" s="284" t="s">
+      <c r="J4" s="280" t="s">
         <v>85</v>
       </c>
-      <c r="K4" s="284"/>
-      <c r="L4" s="284"/>
-      <c r="M4" s="291" t="s">
+      <c r="K4" s="280"/>
+      <c r="L4" s="280"/>
+      <c r="M4" s="287" t="s">
         <v>86</v>
       </c>
-      <c r="N4" s="284" t="s">
+      <c r="N4" s="280" t="s">
         <v>13</v>
       </c>
-      <c r="O4" s="287" t="s">
+      <c r="O4" s="283" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="5" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="286"/>
-      <c r="B5" s="286"/>
-      <c r="C5" s="283"/>
-      <c r="D5" s="282"/>
+      <c r="A5" s="282"/>
+      <c r="B5" s="282"/>
+      <c r="C5" s="293"/>
+      <c r="D5" s="292"/>
       <c r="E5" s="146">
         <v>1</v>
       </c>
@@ -6950,8 +6950,8 @@
       <c r="G5" s="146">
         <v>3</v>
       </c>
-      <c r="H5" s="282"/>
-      <c r="I5" s="290"/>
+      <c r="H5" s="292"/>
+      <c r="I5" s="286"/>
       <c r="J5" s="12">
         <v>1</v>
       </c>
@@ -6961,16 +6961,16 @@
       <c r="L5" s="12">
         <v>3</v>
       </c>
-      <c r="M5" s="292"/>
-      <c r="N5" s="284"/>
-      <c r="O5" s="288"/>
+      <c r="M5" s="288"/>
+      <c r="N5" s="280"/>
+      <c r="O5" s="284"/>
     </row>
     <row r="6" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="170" t="str">
         <f>Paėmimas!B6</f>
         <v>3</v>
       </c>
-      <c r="B6" s="279" t="str">
+      <c r="B6" s="289" t="str">
         <f>Paėmimas!C6</f>
         <v>UAB ,,Ekopartneris", L. Ivinskio g. 65, Kaunas. Katilinė. Taršos šaltinis  Nr. 001.</v>
       </c>
@@ -7019,7 +7019,7 @@
     </row>
     <row r="7" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="32"/>
-      <c r="B7" s="280"/>
+      <c r="B7" s="290"/>
       <c r="C7" s="31"/>
       <c r="D7" s="28"/>
       <c r="E7" s="231"/>
@@ -7039,7 +7039,7 @@
     </row>
     <row r="8" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="32"/>
-      <c r="B8" s="280"/>
+      <c r="B8" s="290"/>
       <c r="C8" s="31"/>
       <c r="D8" s="106"/>
       <c r="E8" s="231"/>
@@ -7059,7 +7059,7 @@
     </row>
     <row r="9" spans="1:16" ht="17" x14ac:dyDescent="0.45">
       <c r="A9" s="32"/>
-      <c r="B9" s="280"/>
+      <c r="B9" s="290"/>
       <c r="C9" s="31">
         <v>2</v>
       </c>
@@ -7096,7 +7096,7 @@
     </row>
     <row r="10" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A10" s="32"/>
-      <c r="B10" s="280"/>
+      <c r="B10" s="290"/>
       <c r="C10" s="31"/>
       <c r="D10" s="106"/>
       <c r="E10" s="231"/>
@@ -7113,7 +7113,7 @@
     </row>
     <row r="11" spans="1:16" ht="17" x14ac:dyDescent="0.45">
       <c r="A11" s="32"/>
-      <c r="B11" s="280"/>
+      <c r="B11" s="290"/>
       <c r="C11" s="31">
         <v>41</v>
       </c>
@@ -7149,7 +7149,7 @@
     </row>
     <row r="12" spans="1:16" ht="30.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A12" s="32"/>
-      <c r="B12" s="280"/>
+      <c r="B12" s="290"/>
       <c r="C12" s="138" t="s">
         <v>41</v>
       </c>
@@ -7185,7 +7185,7 @@
     </row>
     <row r="13" spans="1:16" ht="17" x14ac:dyDescent="0.45">
       <c r="A13" s="32"/>
-      <c r="B13" s="280"/>
+      <c r="B13" s="290"/>
       <c r="C13" s="139" t="s">
         <v>42</v>
       </c>
@@ -7221,7 +7221,7 @@
     </row>
     <row r="14" spans="1:16" ht="17" x14ac:dyDescent="0.45">
       <c r="A14" s="32"/>
-      <c r="B14" s="280"/>
+      <c r="B14" s="290"/>
       <c r="C14" s="139" t="s">
         <v>43</v>
       </c>
@@ -7257,7 +7257,7 @@
     </row>
     <row r="15" spans="1:16" ht="17" x14ac:dyDescent="0.45">
       <c r="A15" s="32"/>
-      <c r="B15" s="280"/>
+      <c r="B15" s="290"/>
       <c r="C15" s="140" t="s">
         <v>44</v>
       </c>
@@ -7293,7 +7293,7 @@
     </row>
     <row r="16" spans="1:16" ht="32.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A16" s="22"/>
-      <c r="B16" s="281"/>
+      <c r="B16" s="291"/>
       <c r="C16" s="31"/>
       <c r="D16" s="109"/>
       <c r="E16" s="21"/>
@@ -7327,6 +7327,11 @@
     </sortState>
   </autoFilter>
   <mergeCells count="14">
+    <mergeCell ref="B6:B16"/>
+    <mergeCell ref="C4:C5"/>
+    <mergeCell ref="D4:D5"/>
+    <mergeCell ref="E4:G4"/>
+    <mergeCell ref="H4:H5"/>
     <mergeCell ref="J4:L4"/>
     <mergeCell ref="C1:F1"/>
     <mergeCell ref="A2:O2"/>
@@ -7336,11 +7341,6 @@
     <mergeCell ref="O4:O5"/>
     <mergeCell ref="I4:I5"/>
     <mergeCell ref="M4:M5"/>
-    <mergeCell ref="B6:B16"/>
-    <mergeCell ref="C4:C5"/>
-    <mergeCell ref="D4:D5"/>
-    <mergeCell ref="E4:G4"/>
-    <mergeCell ref="H4:H5"/>
   </mergeCells>
   <phoneticPr fontId="6" type="noConversion"/>
   <pageMargins left="0.70866141732283472" right="0.70866141732283472" top="0.74803149606299213" bottom="0.74803149606299213" header="0.31496062992125984" footer="0.31496062992125984"/>
@@ -7367,12 +7367,12 @@
   </cols>
   <sheetData>
     <row r="3" spans="1:4" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="293" t="s">
+      <c r="A3" s="243" t="s">
         <v>37</v>
       </c>
-      <c r="B3" s="293"/>
-      <c r="C3" s="293"/>
-      <c r="D3" s="293"/>
+      <c r="B3" s="243"/>
+      <c r="C3" s="243"/>
+      <c r="D3" s="243"/>
     </row>
     <row r="5" spans="1:4" ht="67.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="131" t="s">
@@ -7416,6 +7416,26 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="453e7e53-5eb2-45cf-b2ab-34c867e554b8">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="aa0d983d-359a-438c-9953-3af1a8ac0831" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Dokumentas" ma:contentTypeID="0x010100BAB57CF81AE55C4698AAD22D302297F0" ma:contentTypeVersion="18" ma:contentTypeDescription="Kurkite naują dokumentą." ma:contentTypeScope="" ma:versionID="49ab401eb4052690d2a2629974c22fd6">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="453e7e53-5eb2-45cf-b2ab-34c867e554b8" xmlns:ns3="aa0d983d-359a-438c-9953-3af1a8ac0831" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="ab9969d50e0b13c63bc5bd0499c928dc" ns2:_="" ns3:_="">
     <xsd:import namespace="453e7e53-5eb2-45cf-b2ab-34c867e554b8"/>
@@ -7670,27 +7690,26 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{709F4DDD-DF1A-450D-8BF1-976CA47CFD58}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="453e7e53-5eb2-45cf-b2ab-34c867e554b8"/>
+    <ds:schemaRef ds:uri="aa0d983d-359a-438c-9953-3af1a8ac0831"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="453e7e53-5eb2-45cf-b2ab-34c867e554b8">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="aa0d983d-359a-438c-9953-3af1a8ac0831" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{605DD0A7-BC00-4D8E-8AD3-26E2A9FDEA54}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A0A5B190-5FE3-4B47-B164-68F6A6922F48}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -7707,23 +7726,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{605DD0A7-BC00-4D8E-8AD3-26E2A9FDEA54}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{709F4DDD-DF1A-450D-8BF1-976CA47CFD58}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="453e7e53-5eb2-45cf-b2ab-34c867e554b8"/>
-    <ds:schemaRef ds:uri="aa0d983d-359a-438c-9953-3af1a8ac0831"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>